<commit_message>
finish dairy enteric test
</commit_message>
<xml_diff>
--- a/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
+++ b/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9374AE3A-8F48-4E24-958F-C4F43063A3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C59C64C6-9746-403D-A9DA-6885C9D0B99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1755" yWindow="1020" windowWidth="36255" windowHeight="19140" firstSheet="2" activeTab="5" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1830" yWindow="1065" windowWidth="36255" windowHeight="19140" firstSheet="2" activeTab="5" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -57,7 +57,9 @@
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableNumber">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, IF(ISNUMBER(_xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, "")), _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""), 0))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableOneColumnAndHeader">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue1, _xlpm.LookupArray1, _xlfn.XLOOKUP(_xlpm.LookupValue2, _xlpm.LookupArray2, _xlpm.ReturnArray)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableTwoColumns">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(1, (_xlpm.LookupArray1 = _xlpm.LookupValue1) * (_xlpm.LookupArray2 = _xlpm.LookupValue2), _xlpm.ReturnArray, ""))</definedName>
+    <definedName name="Common_InputFunctions.Utility_ResultsItemFromEquationTitleAndSource">_xlfn.LAMBDA(_xlpm.TitleCell,_xlpm.SourceCell, SUBSTITUTE(LEFT(_xlpm.SourceCell, FIND(",", _xlpm.SourceCell) - 1), "VEERG 2026: ", "") &amp; " " &amp; _xlpm.TitleCell)</definedName>
     <definedName name="Common_InputFunctions.Utility_SourceHyperlink">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#'" &amp; _xlpm.sh &amp; "'!" &amp; _xlpm.addr))</definedName>
+    <definedName name="Common_InputFunctions.Utility_SourceHyperlinkDifferentSheet">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#" &amp; _xlpm.addr))</definedName>
     <definedName name="Common_InputFunctions.Utility_SplitStringIntoArray">_xlfn.LAMBDA(_xlpm.Cell,_xlpm.Delimiter,_xlop.CharacterToRemove1,_xlop.CharacterToRemove2, _xlfn.FILTERXML("&lt;t&gt;&lt;s&gt;" &amp; SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlpm.Cell, _xlpm.CharacterToRemove1, ""), _xlpm.CharacterToRemove2, ""), _xlpm.Delimiter, "&lt;/s&gt;&lt;s&gt;") &amp; "&lt;/s&gt;&lt;/t&gt;", "//s"))</definedName>
     <definedName name="Common_InputFunctions.Utility_SumQuantityFromCriteria">_xlfn.LAMBDA(_xlpm.Criteria1,_xlpm.Criteria1TypeArray,_xlpm.Quantity,_xlop.Multiplier,_xlop.Criteria2,_xlop.Criteria2Array, _xlfn.LET(_xlpm.multiplier, IF(_xlfn.ISOMITTED(_xlpm.Multiplier), 1, _xlpm.Multiplier), _xlpm.quantity, _xlpm.Quantity * _xlpm.multiplier, _xlpm.criteria1, --(_xlpm.Criteria1TypeArray = _xlpm.Criteria1), _xlpm.criteria2, IF(_xlfn.ISOMITTED(_xlpm.Criteria2), 1, --(_xlpm.Criteria2Array = _xlpm.Criteria2)), SUMPRODUCT(_xlpm.criteria1 * _xlpm.criteria2 * _xlpm.quantity)))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State/Territory","Common Name","Abbreviation";"New South Wales","New South Wales","NSW";"Australian Capital Territory","ACT","ACT";"Victoria","Victoria","VIC";"Queensland","Queensland","QLD";"South Australia","South Australia","SA";"Western Australia","Western Australia","WA";"Tasmania","Tasmania","TAS";"Northern Territory","Northern Territory","NT"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -222,6 +224,31 @@
     <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Title">_xlfn.LAMBDA("Table 5.12 Additional symbols used in algorithms for manure related emissions")</definedName>
     <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Vairable">_xlfn.LAMBDA("MMS")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Cattle, for manufacturing beef","Australia";"Cattle, for prime beef","NSW";"Cattle, weaners","NT";"","QLD";"","SA";"","TAS";"","VIC";"","WA"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Title">_xlfn.LAMBDA("Beef cattle products for scope 3")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Unit">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_BeefCattle_Vairable">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Chickens","Australia"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Title">_xlfn.LAMBDA("Chickens products for scope 3")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Unit">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Chickens_Vairable">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Dairy cows","VIC"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Title">_xlfn.LAMBDA("Dairy cattle products for scope 3")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Unit">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Dairycattle_Vairable">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Pigs","Australia"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Title">_xlfn.LAMBDA("Pigs products for scope 3")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Unit">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Pigs_Vairable">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Source region";"Sheep, for mutton","Australia";"Sheep, for prime lamb","NSW";"","QLD";"","SA";"","TAS";"","VIC";"","WA"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Source">_xlfn.LAMBDA("Lifecycles. (2026). Greenhouse Gas Emission Intensities for Material Inputs to Australian Agriculture, Fisheries and Forestry. Version 48. doi 10.5281/zenodo.19656580")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Title">_xlfn.LAMBDA("Sheep products for scope 3")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Unit">_xlfn.LAMBDA("")</definedName>
+    <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Product_Sheep_Vairable">_xlfn.LAMBDA("")</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__1_TotalAnnualMethaneFromEntericFermentation">_xlfn.LAMBDA(_xlpm.N_j124,_xlpm.M_j124,_xlpm.D_j124,_xlpm.N_j35,_xlpm.M_j35,_xlpm.D_j35,_xlpm.MPW_ENTERIC_j35, ((_xlpm.N_j124 * _xlpm.M_j124 * _xlpm.D_j124) + (_xlpm.N_j35 * _xlpm.M_j35 * _xlpm.D_j35) + (_xlpm.N_j35 * _xlpm.MPW_ENTERIC_j35 * _xlpm.D_j35)) * 10 ^ -3)</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__1_TotalAnnualMethaneFromEntericFermentation_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"N_j124","number of dairy cattle in classes j=1,2,4","head","Input";"M_j124","daily enteric methane production for classes j=1,2,4","kg CH4/head/day","Calculated from 3.3.1.1 (2)";"D_j124","duration of stay on the farm for classes j=1,2,4","days","Input";"N_j35","number of dairy cattle in classes j=3,5","head","Input";"M_j35","daily enteric methane production for weaned classes j=3,5","kg CH4/head/day","Calculated from 3.3.1.1 (2)";"D_j35","duration of stay on the farm for weaned classes j=3,5","days","Input";"DPW_j35","duration of stay on the farm for pre-weaned heifer and bull calves","days","Input";"MPW_ENTERIC_j35","daily methane production for pre-weaned heifer and bull calves","kg CH4/head/day","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__1_TotalAnnualMethaneFromEntericFermentation_LatexEquation">_xlfn.LAMBDA("E_{enteric}=\sum\nolimits_j((N_{j=1,2,4}\times M_{j=1,2,4}\times D_{j=1,2,4})+(N_{j=3,5}\times M_{j=3,5}\times D_{j=3,5})+(N_{j=3,5}\times MPW_{ENTERIC,j=3,5}\times D_{j=3,5}))\times 10^{-3}")</definedName>
@@ -259,7 +286,7 @@
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__4_AdditionalIntakeForMilkProduction_Variable">_xlfn.LAMBDA("MI_j")</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__4_AdditionalIntakeForMilkProduction_Variation">_xlfn.LAMBDA("VARATION ON SOURCE: Added milk production unit variable to allow for use of either milk solids or litres of milk.")</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids">_xlfn.LAMBDA(_xlpm.MS_j,_xlpm.FC_j,_xlpm.PC_j, _xlpm.MS_j / (0.01 * (_xlpm.FC_j + _xlpm.PC_j)))</definedName>
-    <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MPU","input milk production unit","","Input";"MS_j","daily production of milk solids","kg MS/head/day","Input";"FC_j","fat content in fat and protein corrected milk","per cent","Constant";"PC_j","protein content in fat and protein corrected milk","per cent","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MPU","input milk production unit","","Input";"MS_j","daily production of milk solids","kg MS/head/day","Input";"FC_j","fat content in fat and protein corrected milk","per cent","Input";"PC_j","protein content in fat and protein corrected milk","per cent","Input"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_Arguments_Method2">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MPU","milk production unit","","Input";"MS_j","daily production of milk solids","kg MS/head/day","Input";"FC_j","fat content in fat and protein corrected milk","per cent","Input";"PC_j","protein content in fat and protein corrected milk","per cent","Input"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_LatexEquation">_xlfn.LAMBDA("MP_j=\frac{MS_j}{0.01\times (FC_j+PC_j)}")</definedName>
     <definedName name="EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_NIRReference">_xlfn.LAMBDA("")</definedName>
@@ -380,6 +407,12 @@
     <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoff_Unit">_xlfn.LAMBDA("Dimensionless")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoff_Variable">_xlfn.LAMBDA("Frac_LEACH_MS")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoff_Variation">_xlfn.LAMBDA("")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoffSolidStorage_Data">_xlfn.LAMBDA(0.02)</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoffSolidStorage_Source">_xlfn.LAMBDA("VEERG 2026: 4.3.2.3 CONSTANTS")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoffSolidStorage_Title">_xlfn.LAMBDA("Fraction of nitrogen lost through leaching and runoff for solid storage MMS only")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoffSolidStorage_Unit">_xlfn.LAMBDA("Fraction")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoffSolidStorage_Variable">_xlfn.LAMBDA("Frac_LEACH_MS")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FractionOfNitrogenLostThroughLeachingAndRunoffSolidStorage_Variation">_xlfn.LAMBDA("")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FractionVolatileSolidsVoidedMMS_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(5, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Area","Pasture","Milking Shed","Feedpad";"System 1: Grazed Only",0.89,0.11,0;"System 2: On feedpad for &lt;10 hr/day for &lt;3 months/year",0.79,0.11,0.1;"System 3: Pasture-grazed 3-9 months/year",0.534,0.11,0.356;"System 4: Zero grazing",0,0.11,0.89}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FractionVolatileSolidsVoidedMMS_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.3.10")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FractionVolatileSolidsVoidedMMS_Title">_xlfn.LAMBDA("Table A.1.3.10: Dairy cattle - Fraction of volatile solids voided to each manure management system (fraction) (MMSjm)")</definedName>
@@ -475,10 +508,6 @@
     <definedName name="X_Cell_Dairy_Breed">'Input - Dairy'!$E$7</definedName>
     <definedName name="X_Cell_Dairy_MilkProductionAmount">'Input - Dairy'!$E$52</definedName>
     <definedName name="X_Cell_Dairy_MilkProductionUnit">'Input - Dairy'!$E$49</definedName>
-    <definedName name="X_Cell_Dairy_MilkSolidsFatContent_Method1">'Input - Dairy'!$E$55</definedName>
-    <definedName name="X_Cell_Dairy_MilkSolidsFatContent_Method2">'Input - Dairy'!$F$55</definedName>
-    <definedName name="X_Cell_Dairy_MilkSolidsProteinContent_Method1">'Input - Dairy'!$F$56</definedName>
-    <definedName name="X_Cell_Dairy_MilkSolidsProteinContent_Method2">'Input - Dairy'!$F$56</definedName>
     <definedName name="X_Cell_Site_AverageTemperature">'Input - Site'!$E$25</definedName>
     <definedName name="X_Cell_Site_ClimateZone">'Input - Site'!$E$31</definedName>
     <definedName name="X_Cell_Site_Elevation">'Input - Site'!$E$24</definedName>
@@ -503,6 +532,7 @@
     <definedName name="X_Table_Dairy_HerdMovement">'Input - Dairy'!$D$9:$I$10</definedName>
     <definedName name="X_Table_Dairy_Liveweight_Method1">'Input - Dairy'!$D$13:$I$15</definedName>
     <definedName name="X_Table_Dairy_Liveweight_Method2">'Input - Dairy'!$D$17:$I$19</definedName>
+    <definedName name="X_Table_Dairy_MilkSolidAttributes">'Input - Dairy'!$D$54:$F$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -10205,7 +10235,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="850" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="836" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -15611,15 +15641,15 @@
         <v>Litres of milk</v>
       </c>
       <c r="M37" s="122" t="str" cm="1">
-        <f t="array" ref="M37:N40">_xlfn.CHOOSECOLS(EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_Arguments(),1,2)</f>
+        <f t="array" ref="M37:N40">_xlfn.CHOOSECOLS(EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_Arguments_Method2(),1,2)</f>
         <v>MPU</v>
       </c>
       <c r="N37" s="121" t="str">
-        <v>input milk production unit</v>
+        <v>milk production unit</v>
       </c>
       <c r="O37" s="123"/>
       <c r="P37" s="122" t="str" cm="1">
-        <f t="array" ref="P37:Q40">_xlfn.CHOOSECOLS(EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_Arguments(),3,4)</f>
+        <f t="array" ref="P37:Q40">_xlfn.CHOOSECOLS(EntericMethane_Dairy_Equations.VEERG_3_3_1_1__5_MilkProductionFromMilkSolids_Arguments_Method2(),3,4)</f>
         <v/>
       </c>
       <c r="Q37" s="120" t="str">
@@ -15671,11 +15701,11 @@
       <c r="G39" s="122" t="str">
         <v>per cent</v>
       </c>
-      <c r="H39" s="118" t="str">
-        <v>Constant</v>
+      <c r="H39" s="120" t="str">
+        <v>Input</v>
       </c>
       <c r="I39" s="122">
-        <f>'Input - Dairy'!$E$55*100</f>
+        <f>INDEX(X_Table_Dairy_MilkSolidAttributes,2,2)*100</f>
         <v>4</v>
       </c>
       <c r="M39" s="122" t="str">
@@ -15688,11 +15718,11 @@
       <c r="P39" s="122" t="str">
         <v>per cent</v>
       </c>
-      <c r="Q39" s="118" t="str">
-        <v>Constant</v>
+      <c r="Q39" s="120" t="str">
+        <v>Input</v>
       </c>
       <c r="R39" s="122">
-        <f>'Input - Dairy'!$F$55*100</f>
+        <f>INDEX(X_Table_Dairy_MilkSolidAttributes,2,3)*100</f>
         <v>4</v>
       </c>
     </row>
@@ -15707,11 +15737,11 @@
       <c r="G40" s="122" t="str">
         <v>per cent</v>
       </c>
-      <c r="H40" s="118" t="str">
-        <v>Constant</v>
+      <c r="H40" s="120" t="str">
+        <v>Input</v>
       </c>
       <c r="I40" s="122">
-        <f>'Input - Dairy'!$E$56*100</f>
+        <f>INDEX(X_Table_Dairy_MilkSolidAttributes,3,2)*100</f>
         <v>3.3000000000000003</v>
       </c>
       <c r="M40" s="122" t="str">
@@ -15724,11 +15754,11 @@
       <c r="P40" s="122" t="str">
         <v>per cent</v>
       </c>
-      <c r="Q40" s="118" t="str">
-        <v>Constant</v>
+      <c r="Q40" s="120" t="str">
+        <v>Input</v>
       </c>
       <c r="R40" s="122">
-        <f>'Input - Dairy'!$F$56*100</f>
+        <f>INDEX(X_Table_Dairy_MilkSolidAttributes,3,3)*100</f>
         <v>3.3000000000000003</v>
       </c>
     </row>
@@ -24678,7 +24708,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAaQB0AGwAZQBDAGUAbABsACwAIABTAG8AdQByAGMAZQBDAGUAbABsACwAXABuACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAEwARQBGAFQAKABTAG8AdQByAGMAZQBDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAXAAiACwAIABTAG8AdQByAGMAZQBDAGUAbABsACkAIAAtADEAKQAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFwAIgAsACAAXAAiAFwAIgApACAAXAB1ADAAMAAyADYAIABcACIAIABcACIAIABcAHUAMAAwADIANgAgAFQAaQB0AGwAZQBDAGUAbABsAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAFwAdQAwADAAMwBlADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAxAC8AKAAxACsAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABDAHIAbwBwAFQAeQBwAGUALAAgAEMAcgBvAHAAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFIAZQBzAGkAZAB1AGUAQwByAG8AcABSAGEAdABpAG8AQQByAHIAYQB5ACkAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4ACwAXABuACAAIAAgACAAKAAxAC0ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAKQAvAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgApADsAXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAFIAZQBzAGkAZAB1AGUAUgBlAG0AbwB2AGUAZABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACwAIABBAG0AbwB1AG4AdABSAGUAbQBvAHYAZQBkACwAXABuACAAIAAgACAAKABBAG0AbwB1AG4AdABSAGUAbQBvAHYAZQBkACoAMQAwAF4AMwApAC8AKABUAG8AdABhAGwAUgBlAHMAaQBkAHUAZQAqADEAMABeADMAKQBcAG4AKQAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABDAG8AdwBzACAAYQBuAGQAIABIAGUAaQBmAGUAcgBzACAAKABXAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFcAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEUAeABjAGwAdQBkAGUAZAAgAFwAdQAwADAAMgA3AFIAZQBmAGUAcgBlAG4AYwBlAFwAdQAwADAAMgA3ACwAIABhAHMAIAB0AGgAZQAgAHYAYQBsAHUAZQAgAGkAcwAgAGMAbwBuAHMAaQBzAHQAZQBuAHQAbAB5ACAAXAB1ADAAMAAyADcARABhAGkAcgB5ACAAQQB1AHMAdAByAGEAbABpAGEAIABbADEAXQBcAHUAMAAwADIANwAgAGEAbgBkACAAaQBzACAAbgBvAHQAIAB1AHMAZQBkACAAaQBuACAAYwBhAGwAYwB1AGwAYQB0AGkAbwBuAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAE0AaQBsAGsAaQBuAGcAIABDAG8AdwBzAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGUAZABpAHUAbQAgAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADUANQAwACwAIAAzADgAMAAsACAAMQA1ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABhAHIAZwBlACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AbABzAHQAZQBpAG4ALQBGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADUAMAAsACAANAA1ADAALAAgADEAOAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBpAGUAcwBpAGEAbgAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANQAwADAALAAgADMANQAwACwAIAAxADQANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQBcACIALAAgADQAMAAwACwAIAAyADcANQAsACAAMQAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBlAHIAcwBlAHkAIABjAHIAbwBzAHMAYgByAGUAZABcACIALAAgADQANQAwACwAIAAzADEANQAsACAAMQAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB5AHIAcwBoAGkAcgBlAFwAIgAsACAANQA0ADAALAAgADMANwA1ACwAIAAxADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAHUAZQByAG4AcwBlAHkAXAAiACwAIAA0ADgAMAAsACAAMwAzADUALAAgADEANAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBvAHcAbgAgAFMAdwBpAHMAcwBcACIALAAgADYAMAAwACwAIAA0ADEANQAsACAAMQA3ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBsAGwAYQB3AGEAcgByAGEALwBBAHUAcwBzAGkAZQAgAFIAZQBkAFwAIgAsACAANQA1ADAALAAgADMANwA1ACwAIAAxADUAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEIAdQBsAGwAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBlAGUAZABcACIALAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAYgByAGUAZQBkAHMAXAAiACwAIAA2ADAAMAAsACAAMgAyADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAFcARwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAMAAuADAAMQA2ACwAIAAwAC4ANgAsACAAMAAuADUANwAsACAAMAAuADEALAAgADAALgA4AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAAUgBlAGYAZQByAGUAbgBjAGUAIAB3AGUAaQBnAGgAdABzACAAKABrAGcAKQAgACgAVwBSAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAAUgBlAGYAZQByAGUAbgBjAGUAIAB3AGUAaQBnAGgAdABzACAAKABrAGcAKQAgACgAVwBSAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFcAUgBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADUALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGUAMQBcACIALAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAYwAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgADUAOQAwACwAIAA1ADkAMAAsACAANQA5ADAALAAgADcANwAwACwAIAA3ADcAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAdABhACAAZgBvAHIAIABwAHIAZQAgAC0AIAB3AGUAYQBuAGUAZAAgAGMAYQBsAHYAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAHQAYQAgAGYAbwByACAAcAByAGUAIAAtACAAdwBlAGEAbgBlAGQAIABjAGEAbAB2AGUAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAFMAagA9ADMALAA1ADsAIABOAFAAVwBqAD0AMwAsADUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAaABlAGEAZABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBDAEgANAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAVgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAAoAFYAUwBqAD0AMwAsADUAKQBcACIALAAgAFwAIgBOAGkAdAByAG8AZwBlAG4AIABFAHgAYwByAGUAdABlAGQAIAAoAE4AUABXAGoAPQAzACwANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwBcAHUAMAAwADMAYwAxAFwAIgAsACAAMAAuADAAMQA3ADYALAAgADAALgAyADYAOAA1ACwAIAAwAC4AMAAxADMANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAXAB1ADAAMAAzAGMAMQBcACIALAAgADAALgAwADIAMAA0ACwAIAAwAC4AMwAwADAAMwAsACAAMAAuADAAMAA5ADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AQwBGAGoAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxADAALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAE4AUwBXAFwAIgAsACAAXAAiAE4AVABcACIALAAgAFwAIgBRAEwARABcACIALAAgAFwAIgBTAEEAXAAiACwAIABcACIAVABBAFMAXAAiACwAIABcACIAVgBJAEMAXAAiACwAIABcACIAVwBBAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALgA3ADIALAAgADAALgA3ADYALAAgADAALgA4ACwAIAAwAC4ANwA4ACwAIAAwAC4ANwA0ACwAIAAwAC4ANgA5ACwAIAAwAC4ANwAzACwAIAAwAC4ANwA2ACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAtACAAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMAA1ACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAHMAIAAoAGEAKQBcACIALAAgADAALgAxADUALAAgADAALgAxADgALAAgADAALgA1ADAALAAgADAALgAyADQALAAgADAALgAxADcALAAgADAALgAxADMALAAgADAALgAxADcALAAgADAALgAxADgALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzACAAYQBuAGQAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzACAAYQBuAGQAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBtADsAIABGAHIAYQBjAEcAQQBTAE0AbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZQB4AGMAcgBlAHQAZQBkACkAXAAiACwAIABcACIARgByAGEAYwBHAEEAUwBNAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMQA0ACAAUABhAHMAdAB1AHIAZQBcACIALAAgADAALAAgADAALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMQAgAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIAAwACwAIAAwAC4AMwA1ACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQA9ADIAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAAgAC0AIABTAHUAbQBwACAAYQBuAGQAIABEAGkAcwBwAGUAcgBzAGEAbABcACIALAAgADAALAAgADAALgAwADcALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMwAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAEQAcgBhAGkAbgBzACAAdABvACAAUABhAGQAZABvAGMAawBcACIALAAgADAALAAgADAALgAyACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMwAgAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAwADUALAAgADAALgAzACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA4ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUABXAEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA4ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUABXAEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAEMAbABhAHMAcwAgAGoAXAAiACwAIABcACIATQBQAFcARQBOAFQARQBSAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBjACAAMQAgAHkAZQBhAHIAXAAiACwAIAAwAC4AMAAxADcANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAYwAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMgAwADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEkAbgBjAHIAZQBhAHMAZQBkACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUgBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABNAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFIAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAEMAbABhAHMAcwAgAGoAXAAiACwAIABcACIATQBSAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzACwAIABhAG4AZAAgAGgAbwB1AHMAZQAgAGMAbwB3AHMAXAAiACwAIAAxAC4AMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAbAAgAG8AdABoAGUAcgAgAGMAYQB0AHQAbABlACAAYwBsAGEAcwBzAGUAcwBcACIALAAgADEALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB2AG8AaQBkAGUAZAAgAHQAbwAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABFAHgAYwBsAHUAZABlAGQAIABcAHUAMAAwADIANwBBAG4AbgB1AGEAbAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHQAaQBtAGUAIABzAHAAZQBuAHQAIABwAGUAcgAgAGEAcgBlAGEAXAB1ADAAMAAyADcAIAByAG8AdwAgAGEAcwAgAHQAaABpAHMAIABpAG4AZgBvAHIAbQBhAHQAaQBvAG4AIABpAHMAIABpAG4AIAB0AGgAZQAgAHQAYQBiAGwAZQAgAHQAaQB0AGwAZQAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcgBlAGEAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBNAGkAbABrAGkAbgBnACAAUwBoAGUAZABcACIALAAgAFwAIgBGAGUAZQBkAHAAYQBkAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADEAOgAgAEcAcgBhAHoAZQBkACAATwBuAGwAeQBcACIALAAgADAALgA4ADkALAAgADAALgAxADEALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAAyADoAIABPAG4AIABmAGUAZQBkAHAAYQBkACAAZgBvAHIAIABcAHUAMAAwADMAYwAxADAAIABoAHIALwBkAGEAeQAgAGYAbwByACAAXAB1ADAAMAAzAGMAMwAgAG0AbwBuAHQAaABzAC8AeQBlAGEAcgBcACIALAAgADAALgA3ADkALAAgADAALgAxADEALAAgADAALgAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAAzADoAIABQAGEAcwB0AHUAcgBlAC0AZwByAGEAegBlAGQAIAAzAC0AOQAgAG0AbwBuAHQAaABzAC8AeQBlAGEAcgBcACIALAAgADAALgA1ADMANAAsACAAMAAuADEAMQAsACAAMAAuADMANQA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAANAA6ACAAWgBlAHIAbwAgAGcAcgBhAHoAaQBuAGcAXAAiACwAIAAwACwAIAAwAC4AMQAxACwAIAAwAC4AOAA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEUARgAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHAAZQByACAATQBNAFMAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEUARgAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHAAZQByACAATQBNAFMAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAG0AKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxACAAQQBuAGUAcgBvAGIAaQBjACAATABhAGcAbwBvAG4AXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADIAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAXAAiACwAIAAwACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADMAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAHMAXAAiACwAIAAwACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0ANAAgAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAGYAbwByACAAZQBhAGMAaAAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuAHAAdQB0ACAAYwBsAGEAcwBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABhAHkAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBvAG4AdgBlAHIAdABlAGQAIABmAHIAZQBlACAAdABlAHgAdAAgAGkAbgAgAGQAbwBjAHUAbQBlAG4AdAAgAHQAbwAgAHQAYQBiAGwAZQAsACAAbQBhAHQAYwBoAGkAbgBnACAAbABpAHYAZQBzAHQAbwBjAGsAIABjAGwAYQBzAHMAIABuAGEAbQBlAHMALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIARAB1AHIAYQB0AGkAbwBuACAAKABwAHIAZQAtAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBlACAAMQAgAHkAZQBhAHIAXAAiACwAIAAzADYANQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGUAIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjACAAMQAgAHkAZQBhAHIAXAAiACwAIAAyADgAMQAsACAAOAA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAFwAbgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAUABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMgBcAHQARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIAMAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQATQBEAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMgBcAHQARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA3ADUAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBcAG4ATgBlAHQAIABlAG4AZQByAGcAeQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkAIAAvACAAawBnACAAbQBpAGwAawBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAwADUANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AFwAbgBHAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAZAByAHkAIABtAGEAdAB0AGUAcgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcARQBDAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEoAIAAvACAAawBnAEQATQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADEAOAAuADQAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBcAG4ARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIAB1AHMAZQAgAG8AZgAgAG0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUAIABlAG4AZQByAGcAeQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYAMAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXABuAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADAAOAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXABuAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAXwBvAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAG0AMwAgAEMASAA0AC8AawBnAFYAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAyADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBfAGwAZQBhAGMAaABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADAAMQAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgBvAHIAIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAIABvAG4AbAB5ACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgBvAHIAIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAIABvAG4AbAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBfAEwARQBBAEMASABfAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAyACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARABlAGYAYQB1AGwAdAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAdwBoAGUAbgAgAG0AYQBuAHUAcgBlACAAaQBzACAAZQB4AGMAcgBlAHQAZQBkACAAdABvACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrACAAKABtAD0AMQA0ACkALgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGUAZgBhAHUAbAB0ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAB3AGgAZQBuACAAbQBhAG4AdQByAGUAIABpAHMAIABlAHgAYwByAGUAdABlAGQAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBfAEwARQBBAEMASABfAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIAB2AG8AbABhAHQAaQBsAGkAegBlAGQAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABmAGEAZQBjAGUAcwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAEcAQQBTAE0AcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIAMQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXABuAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcABlAHIAYwBlAG4AdABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMgAgAEQAQQBUAEEAIAAoAE0ARQBUAEgATwBEACAAMQAgAEEATgBEACAAMgAgAE8AUABUAEkATwBOAFMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0AC4AMAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4AUAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAEMAXwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcABlAHIAYwBlAG4AdABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAzAC4AMwApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMwAuADMAOgAgAEUAbgB0AGUAcgBpAGMAIABNAGUAdABoAGEAbgBlACAALQAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAEUAbgB0AGUAcgBpAGMAIABEAGEAaQByAHkAIABDAGEAdAB0AGwAZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXABuAEUAXwBlAG4AdABlAHIAaQBjAFwAbgB0ACAAQwBIADQAXABuAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9ACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ATgBfAGoAMQAyADQAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMQAsADIALAA0ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADEAMgA0ACAAPQAgAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADEAMgA0ACAAPQAgAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMQAsADIALAA0ACAAKABkAGEAeQBzACkAXABuAE4AXwBqADMANQAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQAgACgAaABlAGEAZAApAFwAbgBNAF8AagAzADUAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBEAF8AagAzADUAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQAgACgAZABhAHkAcwApAFwAbgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAxADIANAAsACAATQBfAGoAMQAyADQALAAgAEQAXwBqADEAMgA0ACwAIABOAF8AagAzADUALAAgAE0AXwBqADMANQAsACAARABfAGoAMwA1ACwAIABNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQAsAFwAbgAgACAAIAAgACgAKABOAF8AagAxADIANAAgACoAIABNAF8AagAxADIANAAgACoAIABEAF8AagAxADIANAApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AXwBqADMANQAgACoAIABEAF8AagAzADUAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQAgACoAIABEAF8AagAzADUAKQApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAEQAUABXAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAUABXAF8AagAzADUAKQApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZQBuAHQAZQByAGkAYwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAEgANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABQAFcAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagAxADIANABcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqADEAMgA0AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqADEAMgA0AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMQAsADIALAA0AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagAzADUAXAAiACwAIABcACIAbgB1AG0AYgBlAHIAIABvAGYAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAHcAZQBhAG4AZQBkACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHcAZQBhAG4AZQBkACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABQAFcAXwBqADMANQBcACIALAAgAFwAIgBkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwBcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAXAAiACwAIABcACIAZABhAGkAbAB5ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AEQAUABXAFwAdQAwADAAMgA3ACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIABhACAAcwBlAHAAYQByAGEAdABlACAAaABhAG4AZABsAGkAbgBnACAAbwBmACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGQAdQByAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAIAAoAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALABcAG4AIAAgACAAIAAyADAALgA3ACAAKgAgAEkAXwBqACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGEAcgBtAGwAZQB5ACAAZQB0ACAAYQBsAC4AIAAoADIAMAAxADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAAzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcAG4ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcAG4AVwBfAGoAIAA9ACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAXABuAEwAVwBHAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgAgACgAawBnAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE0AUgBfAGoAIAA9ACAAaQBuAGMAcgBlAGEAcwBlACAAaQBuACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAZgByAGEAYwB0AGkAbwBuACkAXABuAE0ASQBfAGoAIAA9ACAAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVwBfAGoALAAgAEwAVwBHAF8AagAsACAATQBSAF8AagAsACAATQBJAF8AagAsAFwAbgAgACAAIAAgACgAMQAuADEAOAA1ACAAKwAgADAALgAwADAANAA1ADQAIAAqACAAVwBfAGoAIAAtACAAMAAuADAAMAAwADAAMAAyADYAIAAqACAAVwBfAGoAIABeACAAMgAgACsAIAAwAC4AMwAxADUAIAAqACAATABXAEcAXwBqACkAIABeACAAMgAgACoAIABNAFIAXwBqACAAKwAgAE0ASQBfAGoAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdABcACIALAAgAFwAIgBrAGcAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAFcARwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBSAF8AagBcACIALAAgAFwAIgBpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ASQBfAGoAXAAiACwAIABcACIAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBBAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBNAEkAXwBqAFwAbgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAE0ASQBfAGoAPQAoAE0AUABfAGoAXABcAHQAaQBtAGUAcwAgADEALgAwADMAXABcAHQAaQBtAGUAcwAgAE4ARQApAC8AKABHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagApAFwAbgBNAFAAXwBqACAAPQAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABMAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE4ARQAgAD0AIABuAGUAdAAgAGUAbgBlAHIAZwB5ACAAKABNAEoAIABuAGUAdAAgAGUAbgBlAHIAZwB5AC8AawBnACAAbQBpAGwAawApAFwAbgBHAEUAQwAgAD0AIABnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIAAoAE0ASgAvAGsAZwBEAE0AKQBcAG4AawAgAD0AIABlAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAdQBzAGUAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4AcQBtAF8AagAgAD0AIABtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0ACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBQAF8AagAsACAATgBFACwAIABHAEUAQwAsACAAawAsACAAcQBtAF8AagAsAFwAbgAgACAAIAAgACgATQBQAF8AagAgACoAIAAxAC4AMAAzACAAKgAgAE4ARQApACAALwAgACgARwBFAEMAIAAqACAAawAgACoAIABxAG0AXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagA9AFwAXABmAHIAYQBjAHsATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFAH0AewBHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFUAXAAiACwAIABcACIAaQBuAHAAdQB0ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABfAGoAXAAiACwAIABcACIAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGkAZgAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwApAFwAIgAsACAAXAAiAEwALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBcACIALAAgAFwAIgBuAGUAdAAgAGUAbgBlAHIAZwB5AFwAIgAsACAAXAAiAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBFAEMAXAAiACwAIABcACIAZwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0AFwAIgAsACAAXAAiAE0ASgAvAGsAZwBEAE0AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBrAFwAIgAsACAAXAAiAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBtAF8AagBcACIALAAgAFwAIgBtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADYAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0ACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIAB1AHMAZQAgAG8AZgAgAGUAaQB0AGgAZQByACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAbwByACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4ATQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABjAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBvAG0AIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXABuAE0AUABfAGoAXABuAEwALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AUABfAGoAPQBNAFMAXwBqAC8AKAAwAC4AMAAxAFwAXAB0AGkAbQBlAHMAIAAoAEYAQwBfAGoAKwBQAEMAXwBqACkAKQBcAG4ATQBTAF8AagAgAD0AIABkAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAKABrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARgBDAF8AagAgAD0AIABmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAFAAQwBfAGoAIAA9ACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBTAF8AagAsACAARgBDAF8AagAsACAAUABDAF8AagAsAFwAbgAgACAAIAAgAE0AUwBfAGoAIAAvACAAKAAwAC4AMAAxACAAKgAgACgARgBDAF8AagAgACsAIABQAEMAXwBqACkAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAPQBcAFwAZgByAGEAYwB7AE0AUwBfAGoAfQB7ADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgAgAEMAbwBuAHYAZQByAHQAZQBkACAAaQBuAHAAdQB0ACAARgBDACAAYQBuAGQAIABQAEMAIABwAGUAcgBjAGUAbgB0ACAAdABvACAAaQBuAHQAZQBnAGUAcgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXABuAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIABkAGkAZQB0AFwAbgBxAG0AXwBqAFwAbgBmAHIAYQBjAHQAaQBvAG4AXABuAHEAbQBfAGoAPQAwAC4ANwA5ADUAXABcAHQAaQBtAGUAcwAgACgARABNAEQAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAMAApAC0AMAAuADAAMAAxADQAXABuAEQATQBEAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAE0ARABfAGoALABcAG4AIAAgACAAIAAwAC4ANwA5ADUAIAAqACAAKABEAE0ARABfAGoAIAAqACAAMQAwADAAKQAgAC0AIAAwAC4AMAAwADEANABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQATQBEAF8AagAsAFwAbgAgACAAIAAgADAALgAwADAANwA5ADUAIAAqACAAKABEAE0ARABfAGoAIAAqACAAMQAwADAAKQAgAC0AIAAwAC4AMAAwADEANABcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQAgAG8AZgAgAGQAaQBlAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBxAG0AXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA2ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAPQAwAC4ANwA5ADUAXABcAHQAaQBtAGUAcwAgACgARABNAEQAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAMAApAC0AMAAuADAAMAAxADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgAwADAANwA5ADUAXABcAHQAaQBtAGUAcwAgACgARABNAEQAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAMAApAC0AMAAuADAAMAAxADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQATQBEAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAYwBoAGEAbgBnAGUAZAAgADAALgA3ADkANQAgAHQAbwAgADAALgAwADAANwA5ADUAIAB3AGgAaQBjAGgAIABpAHMAIAB0AGgAZQAgAHYAYQBsAHUAZQAgAHUAcwBlAGQAIABpAG4AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAXAAiACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8ARABhAGkAcgB5ACIALAAiAHQAZQB4AHQAIgA6ACIAQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBNAE0AUwBBAGYAdABlAHIAUwBvAGwAaQBkAFMAZQBwAGEAcgBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABNAE0AUwBGAHIAYQBjAHQAaQBvAG4ALAAgAEYAcgBhAGMAdABpAG8AbgBTAGUAcABhAHIAYQB0AGUAZAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AIAAqACAAKABNAE0AUwBGAHIAYQBjAHQAaQBvAG4ALQAoAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAqAEYAcgBhAGMAdABpAG8AbgBTAGUAcABhAHIAYQB0AGUAZAApACkAXABuACkAOwBcAG4AXABuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAG4AaQB0AGEAbABTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBGAHIAYQBjAHQAaQBvAG4ALABcAG4AIAAgACAAIABNAE0AUwAxAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMQBTAGUAcABhAHIAYQB0AGUAZAAsACAAXABuACAAIAAgACAATQBNAFMAMgBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADIAUwBlAHAAYQByAGEAdABlAGQALAAgAFwAbgAgACAAIAAgAE0ATQBTADMARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAzAFMAZQBwAGEAcgBhAHQAZQBkACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAgACoAIAAoAFwAbgAgACAAIAAgACAAIAAgACAASQBuAGkAdABhAGwAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUARgByAGEAYwB0AGkAbwBuACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACgATQBNAFMAMQBGAHIAYQBjAHQAaQBvAG4AIAAqACAATQBNAFMAMQBTAGUAcABhAHIAYQB0AGUAZAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACgATQBNAFMAMgBGAHIAYQBjAHQAaQBvAG4AIAAqACAATQBNAFMAMgBTAGUAcABhAHIAYQB0AGUAZAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACgATQBNAFMAMwBGAHIAYQBjAHQAaQBvAG4AIAAqACAATQBNAFMAMwBTAGUAcABhAHIAYQB0AGUAZAApAFwAbgAgACAAIAAgACkAXABuACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBSAGUAcwBpAGQAdQBlAFIAZQBtAG8AdgBlAGQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAEQAYQB0AGEAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAF8ATQBlAHQAaABvAGQAMgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8ARABhAGkAcgB5AC4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBNAE0AUwBBAGYAdABlAHIAUwBvAGwAaQBkAFMAZQBwAGEAcgBhAHQAaQBvAG4AIgAsACIASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8ARABhAGkAcgB5AC4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24877,12 +24912,7 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAG4AZAAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIAB0AG8AIAB0AGgAZQAgAHMAbwBpAGwAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAPAB0AD4APABzAD4AXAAiACAAJgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgA8AC8AcwA+ADwAcwA+AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAXAAiADwALwBzAD4APAAvAHQAPgBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAD4APQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApADwAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAD4APQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApADwAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQA+AD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQA8AD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAD4APQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAPAA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQA+AD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAPAA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAD4APQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApADwAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AJwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPABTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAD4ARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgACYAIABcACIAIAB0AG8AIABcACIAIAAmACAAZQBuAGQAcwBUAGUAeAB0ACAAJgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAJwBcACIAIAAmACAAcwBoACAAJgAgAFwAIgAnACEAXAAiACAAJgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0AFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAAiACAAJgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAaQB0AGwAZQBDAGUAbABsACwAIABTAG8AdQByAGMAZQBDAGUAbABsACwAXABuACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAEwARQBGAFQAKABTAG8AdQByAGMAZQBDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAXAAiACwAIABTAG8AdQByAGMAZQBDAGUAbABsACkAIAAtADEAKQAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFwAIgAsACAAXAAiAFwAIgApACAAJgAgAFwAIgAgAFwAIgAgACYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAA+ADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAxAC8AKAAxACsAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABDAHIAbwBwAFQAeQBwAGUALAAgAEMAcgBvAHAAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFIAZQBzAGkAZAB1AGUAQwByAG8AcABSAGEAdABpAG8AQQByAHIAYQB5ACkAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4ACwAXABuACAAIAAgACAAKAAxAC0ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAKQAvAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgApADsAXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAFIAZQBzAGkAZAB1AGUAUgBlAG0AbwB2AGUAZABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACwAIABBAG0AbwB1AG4AdABSAGUAbQBvAHYAZQBkACwAXABuACAAIAAgACAAKABBAG0AbwB1AG4AdABSAGUAbQBvAHYAZQBkACoAMQAwAF4AMwApAC8AKABUAG8AdABhAGwAUgBlAHMAaQBkAHUAZQAqADEAMABeADMAKQBcAG4AKQAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABDAG8AdwBzACAAYQBuAGQAIABIAGUAaQBmAGUAcgBzACAAKABXAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFcAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEUAeABjAGwAdQBkAGUAZAAgACcAUgBlAGYAZQByAGUAbgBjAGUAJwAsACAAYQBzACAAdABoAGUAIAB2AGEAbAB1AGUAIABpAHMAIABjAG8AbgBzAGkAcwB0AGUAbgB0AGwAeQAgACcARABhAGkAcgB5ACAAQQB1AHMAdAByAGEAbABpAGEAIABbADEAXQAnACAAYQBuAGQAIABpAHMAIABuAG8AdAAgAHUAcwBlAGQAIABpAG4AIABjAGEAbABjAHUAbABhAHQAaQBvAG4ALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHIAZQBlAGQAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAD4AMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGUAZABpAHUAbQAgAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADUANQAwACwAIAAzADgAMAAsACAAMQA1ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABhAHIAZwBlACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AbABzAHQAZQBpAG4ALQBGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADUAMAAsACAANAA1ADAALAAgADEAOAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBpAGUAcwBpAGEAbgAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANQAwADAALAAgADMANQAwACwAIAAxADQANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQBcACIALAAgADQAMAAwACwAIAAyADcANQAsACAAMQAxADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBlAHIAcwBlAHkAIABjAHIAbwBzAHMAYgByAGUAZABcACIALAAgADQANQAwACwAIAAzADEANQAsACAAMQAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB5AHIAcwBoAGkAcgBlAFwAIgAsACAANQA0ADAALAAgADMANwA1ACwAIAAxADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAHUAZQByAG4AcwBlAHkAXAAiACwAIAA0ADgAMAAsACAAMwAzADUALAAgADEANAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBvAHcAbgAgAFMAdwBpAHMAcwBcACIALAAgADYAMAAwACwAIAA0ADEANQAsACAAMQA3ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBsAGwAYQB3AGEAcgByAGEALwBBAHUAcwBzAGkAZQAgAFIAZQBkAFwAIgAsACAANQA1ADAALAAgADMANwA1ACwAIAAxADUAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEIAdQBsAGwAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBlAGUAZABcACIALAAgAFwAIgBCAHUAbABsAHMAIAA+ADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAPAAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAbAAgAGIAcgBlAGUAZABzAFwAIgAsACAANgAwADAALAAgADIAMgA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAzADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgAgACgAawBnACkAIAAoAEwAVwBHAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAzADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgAgACgAawBnACkAIAAoAEwAVwBHAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABXAEcAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADUALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAD4AMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAD4AMQBcACIALAAgAFwAIgBCAHUAbABsAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAMAAuADAAMQA2ACwAIAAwAC4ANgAsACAAMAAuADUANwAsACAAMAAuADEALAAgADAALgA4AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAAUgBlAGYAZQByAGUAbgBjAGUAIAB3AGUAaQBnAGgAdABzACAAKABrAGcAKQAgACgAVwBSAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAAUgBlAGYAZQByAGUAbgBjAGUAIAB3AGUAaQBnAGgAdABzACAAKABrAGcAKQAgACgAVwBSAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFcAUgBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADUALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAD4AMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAD4AMQBcACIALAAgAFwAIgBCAHUAbABsAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAANQA5ADAALAAgADUAOQAwACwAIAA1ADkAMAAsACAANwA3ADAALAAgADcANwAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAdABhACAAZgBvAHIAIABwAHIAZQAgAC0AIAB3AGUAYQBuAGUAZAAgAGMAYQBsAHYAZQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBqAD0AMwAsADUAOwAgAE4AUABXAGoAPQAzACwANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBBAG4AaQBtAGEAbAAgAGMAbABhAHMAcwAgAGoAJwAgAGMAbwBsAHUAbQBuACAAaABlAGEAZABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBDAEgANAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAVgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAAoAFYAUwBqAD0AMwAsADUAKQBcACIALAAgAFwAIgBOAGkAdAByAG8AZwBlAG4AIABFAHgAYwByAGUAdABlAGQAIAAoAE4AUABXAGoAPQAzACwANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwA8ADEAXAAiACwAIAAwAC4AMAAxADcANgAsACAAMAAuADIANgA4ADUALAAgADAALgAwADEAMwA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwA8ADEAXAAiACwAIAAwAC4AMAAyADAANAAsACAAMAAuADMAMAAwADMALAAgADAALgAwADAAOQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADYAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AQwBGAHMAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBqAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADYAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AQwBGAHMAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBqAG0AKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEMARgBqAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAAnAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEAMAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBUAEEAUwBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAuADcAMgAsACAAMAAuADcANgAsACAAMAAuADgALAAgADAALgA3ADgALAAgADAALgA3ADQALAAgADAALgA2ADkALAAgADAALgA3ADMALAAgADAALgA3ADYALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwAgACgAYQApAFwAIgAsACAAMAAuADEANQAsACAAMAAuADEAOAAsACAAMAAuADUAMAAsACAAMAAuADIANAAsACAAMAAuADEANwAsACAAMAAuADEAMwAsACAAMAAuADEANwAsACAAMAAuADEAOAAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAG0AOwAgAEYAcgBhAGMARwBBAFMATQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZQB4AGMAcgBlAHQAZQBkACkAXAAiACwAIABcACIARgByAGEAYwBHAEEAUwBNAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMQA0ACAAUABhAHMAdAB1AHIAZQBcACIALAAgADAALAAgADAALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMQAgAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIAAwACwAIAAwAC4AMwA1ACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQA9ADIAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAAgAC0AIABTAHUAbQBwACAAYQBuAGQAIABEAGkAcwBwAGUAcgBzAGEAbABcACIALAAgADAALAAgADAALgAwADcALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMwAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAEQAcgBhAGkAbgBzACAAdABvACAAUABhAGQAZABvAGMAawBcACIALAAgADAALAAgADAALgAyACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMwAgAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAwADUALAAgADAALgAzACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA4ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUABXAEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA4ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUABXAEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAEMAbABhAHMAcwAgAGoAXAAiACwAIABcACIATQBQAFcARQBOAFQARQBSAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwAgADwAIAAxACAAeQBlAGEAcgBcACIALAAgADAALgAwADEANwA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgADwAIAAxACAAeQBlAGEAcgBcACIALAAgADAALgAwADIAMAA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA5ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABJAG4AYwByAGUAYQBzAGUAZAAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAIAAoAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQApACAAKABNAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEkAbgBjAHIAZQBhAHMAZQBkACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgATQBSAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABDAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAE0AUgBqAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAYwBvAHcAcwAsACAAYQBuAGQAIABoAG8AdQBzAGUAIABjAG8AdwBzAFwAIgAsACAAMQAuADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBsAGwAIABvAHQAaABlAHIAIABjAGEAdAB0AGwAZQAgAGMAbABhAHMAcwBlAHMAXAAiACwAIAAxAC4AMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB2AG8AaQBkAGUAZAAgAHQAbwAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAGoAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAdgBvAGkAZABlAGQAIAB0AG8AIABlAGEAYwBoACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAE0AUwBqAG0AKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAGoAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAJwBBAG4AbgB1AGEAbAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHQAaQBtAGUAIABzAHAAZQBuAHQAIABwAGUAcgAgAGEAcgBlAGEAJwAgAHIAbwB3ACAAYQBzACAAdABoAGkAcwAgAGkAbgBmAG8AcgBtAGEAdABpAG8AbgAgAGkAcwAgAGkAbgAgAHQAaABlACAAdABhAGIAbABlACAAdABpAHQAbABlAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQByAGUAYQBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE0AaQBsAGsAaQBuAGcAIABTAGgAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAcABhAGQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMQA6ACAARwByAGEAegBlAGQAIABPAG4AbAB5AFwAIgAsACAAMAAuADgAOQAsACAAMAAuADEAMQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADIAOgAgAE8AbgAgAGYAZQBlAGQAcABhAGQAIABmAG8AcgAgADwAMQAwACAAaAByAC8AZABhAHkAIABmAG8AcgAgADwAMwAgAG0AbwBuAHQAaABzAC8AeQBlAGEAcgBcACIALAAgADAALgA3ADkALAAgADAALgAxADEALAAgADAALgAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAAzADoAIABQAGEAcwB0AHUAcgBlAC0AZwByAGEAegBlAGQAIAAzAC0AOQAgAG0AbwBuAHQAaABzAC8AeQBlAGEAcgBcACIALAAgADAALgA1ADMANAAsACAAMAAuADEAMQAsACAAMAAuADMANQA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAANAA6ACAAWgBlAHIAbwAgAGcAcgBhAHoAaQBuAGcAXAAiACwAIAAwACwAIAAwAC4AMQAxACwAIAAwAC4AOAA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEUARgAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHAAZQByACAATQBNAFMAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEUARgAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHAAZQByACAATQBNAFMAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAG0AKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAAnAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBFAEYAbQBcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMQA0ACAAUABhAHMAdAB1AHIAZQBcACIALAAgADAALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMQAgAEEAbgBlAHIAbwBiAGkAYwAgAEwAYQBnAG8AbwBuAFwAIgAsACAAMAAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAyACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAOgAgAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAOgAgAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBzAFwAIgAsACAAMAAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADQAIABTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAMAAuADAAMAA1ACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBcAG4ARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAGYAbwByACAAZQBhAGMAaAAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuAHAAdQB0ACAAYwBsAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABmAG8AcgAgAGUAYQBjAGgAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgBwAHUAdAAgAGMAbABhAHMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGQAYQB5AHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMgBcAHQARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEMAbwBuAHYAZQByAHQAZQBkACAAZgByAGUAZQAgAHQAZQB4AHQAIABpAG4AIABkAG8AYwB1AG0AZQBuAHQAIAB0AG8AIAB0AGEAYgBsAGUALAAgAG0AYQB0AGMAaABpAG4AZwAgAGwAaQB2AGUAcwB0AG8AYwBrACAAYwBsAGEAcwBzACAAbgBhAG0AZQBzAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMwAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAGMAbABhAHMAcwAgAGoAXAAiACwAIABcACIARAB1AHIAYQB0AGkAbwBuACAAKAB3AGUAYQBuAGUAZAApAFwAIgAsACAAXAAiAEQAdQByAGEAdABpAG8AbgAgACgAcAByAGUALQB3AGUAYQBuAGUAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAYwBvAHcAcwBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIAA+ACAAMQAgAHkAZQBhAHIAXAAiACwAIAAzADYANQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMgA4ADEALAAgADgANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAIAA+ACAAMQAgAHkAZQBhAHIAXAAiACwAIAAzADYANQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAIAA8ACAAMQAgAHkAZQBhAHIAXAAiACwAIAAyADgAMQAsACAAOAA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAFwAbgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAUABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMgBcAHQARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIAMAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQATQBEAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMgBcAHQARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA3ADUAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBcAG4ATgBlAHQAIABlAG4AZQByAGcAeQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkAIAAvACAAawBnACAAbQBpAGwAawBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAwADUANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AFwAbgBHAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAZAByAHkAIABtAGEAdAB0AGUAcgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcARQBDAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEoAIAAvACAAawBnAEQATQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADEAOAAuADQAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBcAG4ARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIAB1AHMAZQAgAG8AZgAgAG0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUAIABlAG4AZQByAGcAeQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYAMAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXABuAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADAAOAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXABuAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAXwBvAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAG0AMwAgAEMASAA0AC8AawBnAFYAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAyADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBfAGwAZQBhAGMAaABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADAAMQAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgBvAHIAIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAIABvAG4AbAB5ACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgBvAHIAIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAIABvAG4AbAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBfAEwARQBBAEMASABfAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAyACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARABlAGYAYQB1AGwAdAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAdwBoAGUAbgAgAG0AYQBuAHUAcgBlACAAaQBzACAAZQB4AGMAcgBlAHQAZQBkACAAdABvACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrACAAKABtAD0AMQA0ACkALgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGUAZgBhAHUAbAB0ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAB3AGgAZQBuACAAbQBhAG4AdQByAGUAIABpAHMAIABlAHgAYwByAGUAdABlAGQAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBfAEwARQBBAEMASABfAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIAB2AG8AbABhAHQAaQBsAGkAegBlAGQAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABmAGEAZQBjAGUAcwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAEcAQQBTAE0AcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIAMQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXABuAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcABlAHIAYwBlAG4AdABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMgAgAEQAQQBUAEEAIAAoAE0ARQBUAEgATwBEACAAMQAgAEEATgBEACAAMgAgAE8AUABUAEkATwBOAFMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0AC4AMAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4AUAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAEMAXwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcABlAHIAYwBlAG4AdABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAzAC4AMwApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMwAuADMAOgAgAEUAbgB0AGUAcgBpAGMAIABNAGUAdABoAGEAbgBlACAALQAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAEUAbgB0AGUAcgBpAGMAIABEAGEAaQByAHkAIABDAGEAdAB0AGwAZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXABuAEUAXwBlAG4AdABlAHIAaQBjAFwAbgB0ACAAQwBIADQAXABuAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9ACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ATgBfAGoAMQAyADQAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMQAsADIALAA0ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADEAMgA0ACAAPQAgAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADEAMgA0ACAAPQAgAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMQAsADIALAA0ACAAKABkAGEAeQBzACkAXABuAE4AXwBqADMANQAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQAgACgAaABlAGEAZAApAFwAbgBNAF8AagAzADUAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBEAF8AagAzADUAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQAgACgAZABhAHkAcwApAFwAbgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAxADIANAAsACAATQBfAGoAMQAyADQALAAgAEQAXwBqADEAMgA0ACwAIABOAF8AagAzADUALAAgAE0AXwBqADMANQAsACAARABfAGoAMwA1ACwAIABNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQAsAFwAbgAgACAAIAAgACgAKABOAF8AagAxADIANAAgACoAIABNAF8AagAxADIANAAgACoAIABEAF8AagAxADIANAApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AXwBqADMANQAgACoAIABEAF8AagAzADUAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQAgACoAIABEAF8AagAzADUAKQApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAEQAUABXAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAUABXAF8AagAzADUAKQApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZQBuAHQAZQByAGkAYwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAEgANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABQAFcAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagAxADIANABcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqADEAMgA0AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqADEAMgA0AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMQAsADIALAA0AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagAzADUAXAAiACwAIABcACIAbgB1AG0AYgBlAHIAIABvAGYAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAHcAZQBhAG4AZQBkACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHcAZQBhAG4AZQBkACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABQAFcAXwBqADMANQBcACIALAAgAFwAIgBkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwBcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAXAAiACwAIABcACIAZABhAGkAbAB5ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcARABQAFcAJwAgAHYAYQByAGkAYQBiAGwAZQAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAYQAgAHMAZQBwAGEAcgBhAHQAZQAgAGgAYQBuAGQAbABpAG4AZwAgAG8AZgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABkAHUAcgBhAHQAaQBvAG4ALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcAG4ATQBfAGoAXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AagA9ADIAMAAuADcAXABcAHQAaQBtAGUAcwAgAEkAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBJAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEkAXwBqACwAXABuACAAIAAgACAAMgAwAC4ANwAgACoAIABJAF8AagAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAaABhAHIAbQBsAGUAeQAgAGUAdAAgAGEAbAAuACAAKAAyADAAMQA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AagA9ADIAMAAuADcAXABcAHQAaQBtAGUAcwAgAEkAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAFwAbgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXABuAEkAXwBqAFwAbgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAEkAXwBqAD0AKAAxAC4AMQA4ADUAKwAwAC4AMAAwADQANQA0AFwAXAB0AGkAbQBlAHMAIABXAF8AagAtADAALgAwADAAMAAwADAAMgA2AFwAXAB0AGkAbQBlAHMAIABXAF8AagBeADIAKwAwAC4AMwAxADUAXABcAHQAaQBtAGUAcwAgAEwAVwBHAF8AagApAF4AMgBcAFwAdABpAG0AZQBzACAATQBSAF8AagArAE0ASQBfAGoAXABuAFcAXwBqACAAPQAgAGwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApAFwAbgBMAFcARwBfAGoAIAA9ACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBNAFIAXwBqACAAPQAgAGkAbgBjAHIAZQBhAHMAZQAgAGkAbgAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgBNAEkAXwBqACAAPQAgAGEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFcAXwBqACwAIABMAFcARwBfAGoALAAgAE0AUgBfAGoALAAgAE0ASQBfAGoALABcAG4AIAAgACAAIAAoADEALgAxADgANQAgACsAIAAwAC4AMAAwADQANQA0ACAAKgAgAFcAXwBqACAALQAgADAALgAwADAAMAAwADAAMgA2ACAAKgAgAFcAXwBqACAAXgAgADIAIAArACAAMAAuADMAMQA1ACAAKgAgAEwAVwBHAF8AagApACAAXgAgADIAIAAqACAATQBSAF8AagAgACsAIABNAEkAXwBqAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAzACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAXwBqAD0AKAAxAC4AMQA4ADUAKwAwAC4AMAAwADQANQA0AFwAXAB0AGkAbQBlAHMAIABXAF8AagAtADAALgAwADAAMAAwADAAMgA2AFwAXAB0AGkAbQBlAHMAIABXAF8AagBeADIAKwAwAC4AMwAxADUAXABcAHQAaQBtAGUAcwAgAEwAVwBHAF8AagApAF4AMgBcAFwAdABpAG0AZQBzACAATQBSAF8AagArAE0ASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAXwBqAFwAIgAsACAAXAAiAGwAaQB2AGUAdwBlAGkAZwBoAHQAXAAiACwAIABcACIAawBnAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABXAEcAXwBqAFwAIgAsACAAXAAiAGwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUgBfAGoAXAAiACwAIABcACIAaQBuAGMAcgBlAGEAcwBlACAAaQBuACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEkAXwBqAFwAIgAsACAAXAAiAGEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AQQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ATQBJAF8AagBcAG4AawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAEkAXwBqAD0AKABNAFAAXwBqAFwAXAB0AGkAbQBlAHMAIAAxAC4AMAAzAFwAXAB0AGkAbQBlAHMAIABOAEUAKQAvACgARwBFAEMAXABcAHQAaQBtAGUAcwAgAGsAXABcAHQAaQBtAGUAcwAgAHEAbQBfAGoAKQBcAG4ATQBQAF8AagAgAD0AIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgATAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBOAEUAIAA9ACAAbgBlAHQAIABlAG4AZQByAGcAeQAgACgATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAvAGsAZwAgAG0AaQBsAGsAKQBcAG4ARwBFAEMAIAA9ACAAZwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAKABNAEoALwBrAGcARABNACkAXABuAGsAIAA9ACAAZQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAG0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUAIABlAG4AZQByAGcAeQAgAHUAcwBlACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAZgByAGEAYwB0AGkAbwBuACkAXABuAHEAbQBfAGoAIAA9ACAAbQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQAgAG8AZgAgAHQAaABlACAAZABpAGUAdAAgACgAZgByAGEAYwB0AGkAbwBuACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AUABfAGoALAAgAE4ARQAsACAARwBFAEMALAAgAGsALAAgAHEAbQBfAGoALABcAG4AIAAgACAAIAAoAE0AUABfAGoAIAAqACAAMQAuADAAMwAgACoAIABOAEUAKQAgAC8AIAAoAEcARQBDACAAKgAgAGsAIAAqACAAcQBtAF8AagApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANAApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASQBfAGoAPQBcAFwAZgByAGEAYwB7AE0AUABfAGoAXABcAHQAaQBtAGUAcwAgADEALgAwADMAXABcAHQAaQBtAGUAcwAgAE4ARQB9AHsARwBFAEMAXABcAHQAaQBtAGUAcwAgAGsAXABcAHQAaQBtAGUAcwAgAHEAbQBfAGoAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAGkAbgBwAHUAdAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABfAGoAXAAiACwAIABcACIAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGkAZgAgAGkAbgBwAHUAdAAgAGEAcwAgAGwAaQB0AHIAZQBzACAAbwBmACAAbQBpAGwAawApAFwAIgAsACAAXAAiAEwALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAXwBqAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABpAGYAIABpAG4AcAB1AHQAIABhAHMAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAKQBcACIALAAgAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEUAXAAiACwAIABcACIAbgBlAHQAIABlAG4AZQByAGcAeQBcACIALAAgAFwAIgBNAEoAIABuAGUAdAAgAGUAbgBlAHIAZwB5AC8AawBnACAAbQBpAGwAawBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcARQBDAFwAIgAsACAAXAAiAGcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdABcACIALAAgAFwAIgBNAEoALwBrAGcARABNAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAawBcACIALAAgAFwAIgBlAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAdQBzAGUAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHEAbQBfAGoAXAAiACwAIABcACIAbQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQAgAG8AZgAgAHQAaABlACAAZABpAGUAdABcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA2ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdAAgAHYAYQByAGkAYQBiAGwAZQAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAdQBzAGUAIABvAGYAIABlAGkAdABoAGUAcgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwAgAG8AcgAgAGwAaQB0AHIAZQBzACAAbwBmACAAbQBpAGwAawAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXABuAE0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAYwBvAG4AdgBlAHIAdABlAGQAIABmAHIAbwBtACAAbQBpAGwAawAgAHMAbwBsAGkAZABzAFwAbgBNAFAAXwBqAFwAbgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAFAAXwBqAD0ATQBTAF8AagAvACgAMAAuADAAMQBcAFwAdABpAG0AZQBzACAAKABGAEMAXwBqACsAUABDAF8AagApACkAXABuAE0AUwBfAGoAIAA9ACAAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwAgACgAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEYAQwBfAGoAIAA9ACAAZgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAIAAoAHAAZQByACAAYwBlAG4AdAApAFwAbgBQAEMAXwBqACAAPQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAIAAoAHAAZQByACAAYwBlAG4AdAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AUwBfAGoALAAgAEYAQwBfAGoALAAgAFAAQwBfAGoALABcAG4AIAAgACAAIABNAFMAXwBqACAALwAgACgAMAAuADAAMQAgACoAIAAoAEYAQwBfAGoAIAArACAAUABDAF8AagApACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABjAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBvAG0AIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAXwBqAD0AXABcAGYAcgBhAGMAewBNAFMAXwBqAH0AewAwAC4AMAAxAFwAXAB0AGkAbQBlAHMAIAAoAEYAQwBfAGoAKwBQAEMAXwBqACkAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFUAXAAiACwAIABcACIAaQBuAHAAdQB0ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBTAF8AagBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBpAGwAawAgAHMAbwBsAGkAZABzAFwAIgAsACAAXAAiAGsAZwAgAE0AUwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAQwBfAGoAXAAiACwAIABcACIAZgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABDAF8AagBcACIALAAgAFwAIgBwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAF8ATQBlAHQAaABvAGQAMgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFUAXAAiACwAIABcACIAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBTAF8AagBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBpAGwAawAgAHMAbwBsAGkAZABzAFwAIgAsACAAXAAiAGsAZwAgAE0AUwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAQwBfAGoAXAAiACwAIABcACIAZgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABDAF8AagBcACIALAAgAFwAIgBwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0ACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIAB1AHMAZQAgAG8AZgAgAGUAaQB0AGgAZQByACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAbwByACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrAC4AIABDAG8AbgB2AGUAcgB0AGUAZAAgAGkAbgBwAHUAdAAgAEYAQwAgAGEAbgBkACAAUABDACAAcABlAHIAYwBlAG4AdAAgAHQAbwAgAGkAbgB0AGUAZwBlAHIALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFwAbgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcAG4AcQBtAF8AagBcAG4AZgByAGEAYwB0AGkAbwBuAFwAbgBxAG0AXwBqAD0AMAAuADcAOQA1AFwAXAB0AGkAbQBlAHMAIAAoAEQATQBEAF8AagBcAFwAdABpAG0AZQBzACAAMQAwADAAKQAtADAALgAwADAAMQA0AFwAbgBEAE0ARABfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAIABlAHgAcAByAGUAcwBzAGUAZAAgAGEAcwAgAGEAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABNAEQAXwBqACwAXABuACAAIAAgACAAMAAuADcAOQA1ACAAKgAgACgARABNAEQAXwBqACAAKgAgADEAMAAwACkAIAAtACAAMAAuADAAMAAxADQAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAE0ARABfAGoALABcAG4AIAAgACAAIAAwAC4AMAAwADcAOQA1ACAAKgAgACgARABNAEQAXwBqACAAKgAgADEAMAAwACkAIAAtACAAMAAuADAAMAAxADQAXABuACAAIAApADsAXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIABkAGkAZQB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBxAG0AXwBqAD0AMAAuADcAOQA1AFwAXAB0AGkAbQBlAHMAIAAoAEQATQBEAF8AagBcAFwAdABpAG0AZQBzACAAMQAwADAAKQAtADAALgAwADAAMQA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAPQAwAC4AMAAwADcAOQA1AFwAXAB0AGkAbQBlAHMAIAAoAEQATQBEAF8AagBcAFwAdABpAG0AZQBzACAAMQAwADAAKQAtADAALgAwADAAMQA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAE0ARABfAGoAXAAiACwAIABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAIABlAHgAcAByAGUAcwBzAGUAZAAgAGEAcwAgAGEAIABmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAGMAaABhAG4AZwBlAGQAIAAwAC4ANwA5ADUAIAB0AG8AIAAwAC4AMAAwADcAOQA1ACAAdwBoAGkAYwBoACAAaQBzACAAdABoAGUAIAB2AGEAbAB1AGUAIAB1AHMAZQBkACAAaQBuACAAdABoAGUAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0AFwAIgApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAATQBNAFMARgByAGEAYwB0AGkAbwBuACwAIABGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgATQBNAFMARgByAGEAYwB0AGkAbwBuAC0AKABNAE0AUwBGAHIAYQBjAHQAaQBvAG4AKgBGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQAKQApAFwAbgApADsAXABuAFwAbgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQBuAGkAdABhAGwAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUARgByAGEAYwB0AGkAbwBuACwAXABuACAAIAAgACAATQBNAFMAMQBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQALAAgAFwAbgAgACAAIAAgAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMwBTAGUAcABhAHIAYQB0AGUAZAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AIAAqACAAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADIAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADMARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEIAZQBlAGYAQwBhAHQAdABsAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEIAZQBlAGYAQwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEIAZQBlAGYAQwBhAHQAdABsAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEIAZQBlAGYAQwBhAHQAdABsAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBSAGUAcwBpAGQAdQBlAFIAZQBtAG8AdgBlAGQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAEQAYQB0AGEAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAF8ATQBlAHQAaABvAGQAMgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8ARABhAGkAcgB5AC4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBNAE0AUwBBAGYAdABlAHIAUwBvAGwAaQBkAFMAZQBwAGEAcgBhAHQAaQBvAG4AIgAsACIASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8ARABhAGkAcgB5AC4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24897,9 +24927,9 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -24924,9 +24954,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
dairy enterprise wip, excel hygine scripts
</commit_message>
<xml_diff>
--- a/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
+++ b/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE600743-6972-4F4A-859B-836E35DCB13A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A577E809-35B0-4AA4-9BE9-ABBB9AC9475E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" firstSheet="7" activeTab="7" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="2085" yWindow="1230" windowWidth="36255" windowHeight="19140" activeTab="5" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="3.3.1.1-2 Enteric Methane" sheetId="69" r:id="rId6"/>
     <sheet name="Constants - Dairy" sheetId="79" r:id="rId7"/>
     <sheet name="Constants - Common" sheetId="110" r:id="rId8"/>
-    <sheet name="Constants - Livestock" sheetId="43" r:id="rId9"/>
+    <sheet name="Constants - Common Livestock" sheetId="43" r:id="rId9"/>
     <sheet name="Acknowledgements" sheetId="72" r:id="rId10"/>
   </sheets>
   <definedNames>
@@ -642,7 +642,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="254">
   <si>
     <t>INPUTS</t>
   </si>
@@ -1474,6 +1474,15 @@
   </si>
   <si>
     <t>EFNi &amp; EFN2Oi</t>
+  </si>
+  <si>
+    <t>Livestock classes</t>
+  </si>
+  <si>
+    <t>Table_LivestockClasses_Dairy</t>
+  </si>
+  <si>
+    <t>Livestock class</t>
   </si>
 </sst>
 </file>
@@ -3586,32 +3595,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -4473,6 +4456,32 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -9215,7 +9224,7 @@
   </autoFilter>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{F2B173A3-CADE-4DCA-988D-39EE2392D8DB}" name="MMS"/>
-    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="43" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="79" dataCellStyle="Content normal"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9233,13 +9242,13 @@
     <tableColumn id="1" xr3:uid="{8ACEF380-8A1A-411E-A23A-665A769E20C7}" name="MMS m">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_NitrousOxideEFsAndFracGASM_Data(), Table_SourceData_Dairy_EFmFracGASM[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1898B440-928B-49CE-BE96-215FD9903B4D}" name="EFm" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{1898B440-928B-49CE-BE96-215FD9903B4D}" name="EFm" dataDxfId="54" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_NitrousOxideEFsAndFracGASM_Data(), Table_SourceData_Dairy_EFmFracGASM[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E38469E4-0572-4872-BE43-36C7BBE75007}" name="FracGASMm" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{E38469E4-0572-4872-BE43-36C7BBE75007}" name="FracGASMm" dataDxfId="53" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_NitrousOxideEFsAndFracGASM_Data(), Table_SourceData_Dairy_EFmFracGASM[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2136786A-A3D3-4E62-B5A7-46AAC51855AD}" name="NIR reference" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{2136786A-A3D3-4E62-B5A7-46AAC51855AD}" name="NIR reference" dataDxfId="52" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_NitrousOxideEFsAndFracGASM_Data(), Table_SourceData_Dairy_EFmFracGASM[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9257,7 +9266,7 @@
     <tableColumn id="1" xr3:uid="{34872B36-E9B0-443E-A8EC-EC35C2572085}" name="Animal class j">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MethaneProductionPreWeanedCalves_Data(), Table_SourceData_Dairy_MPWENTERIC[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5BF46DC3-A57C-4E83-B386-D48BB1DB64E1}" name="MPW ENTERIC" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{5BF46DC3-A57C-4E83-B386-D48BB1DB64E1}" name="MPW ENTERIC" dataDxfId="51" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MethaneProductionPreWeanedCalves_Data(), Table_SourceData_Dairy_MPWENTERIC[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9275,7 +9284,7 @@
     <tableColumn id="1" xr3:uid="{B2383F7B-29D1-4559-9E34-4E2C127CFB5C}" name="Animal class j">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_IncreasedMetabolicRateMilk_Data(), Table_SourceData_Dairy_MRj[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D1C6DB76-173B-4192-987A-A32F6D0D0E1A}" name="MRj" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{D1C6DB76-173B-4192-987A-A32F6D0D0E1A}" name="MRj" dataDxfId="50" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_IncreasedMetabolicRateMilk_Data(), Table_SourceData_Dairy_MRj[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9295,13 +9304,13 @@
     <tableColumn id="1" xr3:uid="{A4A196FD-DBDB-46C0-83CE-7C77F2C477B3}" name="Area">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_FractionVolatileSolidsVoidedMMS_Data(), Table_SourceData_Dairy_ProductionSystemTemplates[[#Headers],[Area]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{53A25CAD-C5FE-4619-A71E-7D4EE15E4A88}" name="Pasture" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{53A25CAD-C5FE-4619-A71E-7D4EE15E4A88}" name="Pasture" dataDxfId="49" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_FractionVolatileSolidsVoidedMMS_Data(), Table_SourceData_Dairy_ProductionSystemTemplates[[#Headers],[Area]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9DFD752F-089A-45B1-A1B3-329B65BC5650}" name="Milking shed" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{9DFD752F-089A-45B1-A1B3-329B65BC5650}" name="Milking shed" dataDxfId="48" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_FractionVolatileSolidsVoidedMMS_Data(), Table_SourceData_Dairy_ProductionSystemTemplates[[#Headers],[Area]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{37872FA9-DEFB-4D6F-848C-F92D7B048A75}" name="Feedpad" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{37872FA9-DEFB-4D6F-848C-F92D7B048A75}" name="Feedpad" dataDxfId="47" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_FractionVolatileSolidsVoidedMMS_Data(), Table_SourceData_Dairy_ProductionSystemTemplates[[#Headers],[Area]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9320,10 +9329,10 @@
     <tableColumn id="1" xr3:uid="{D85FDEBC-2FC0-45F1-BCD6-4464E2C22E94}" name="MMS m">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_EFNitrousOxidePerMMS_Data(), Table_SourceData_Dairy_EFm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A21A17E4-5CBE-457C-83F6-E66794AB20C1}" name="EFm" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{A21A17E4-5CBE-457C-83F6-E66794AB20C1}" name="EFm" dataDxfId="46" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_EFNitrousOxidePerMMS_Data(), Table_SourceData_Dairy_EFm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0552581B-C2BB-481C-87D1-7C1129F487A9}" name="NIR reference" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{0552581B-C2BB-481C-87D1-7C1129F487A9}" name="NIR reference" dataDxfId="45" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_EFNitrousOxidePerMMS_Data(), Table_SourceData_Dairy_EFm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9342,10 +9351,10 @@
     <tableColumn id="1" xr3:uid="{C1D0CE9E-4549-48D9-9C0F-1310FC73ABC5}" name="Animal class j">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_DurationOfStay_Data(), Table_SourceData_Dairy_Duration[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1396CED3-63B3-4B3F-8629-5350DAE232F8}" name="Duration (weaned)" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{1396CED3-63B3-4B3F-8629-5350DAE232F8}" name="Duration (weaned)" dataDxfId="44" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_DurationOfStay_Data(), Table_SourceData_Dairy_Duration[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9A35A34C-C373-43B3-B087-AB054A306734}" name="Duration (pre-weaned)" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{9A35A34C-C373-43B3-B087-AB054A306734}" name="Duration (pre-weaned)" dataDxfId="43" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_DurationOfStay_Data(), Table_SourceData_Dairy_Duration[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9354,6 +9363,18 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{E4C31AD6-8635-4CF8-893C-3B663307234C}" name="Table_LivestockClasses_Dairy" displayName="Table_LivestockClasses_Dairy" ref="L7:L12" totalsRowShown="0">
+  <autoFilter ref="L7:L12" xr:uid="{E4C31AD6-8635-4CF8-893C-3B663307234C}">
+    <filterColumn colId="0" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{C3130FCF-5C39-4259-ADC1-C2908930D6B5}" name="Livestock class"/>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{8967E236-752F-4A25-975B-400E88D49496}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
   <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9375,7 +9396,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{3C1AFC1E-172F-4583-853A-ED2A66CBA5A6}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
   <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9389,7 +9410,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{DCA9E2FE-855B-409F-9561-D2BB52D66C11}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9407,7 +9428,21 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B6F3FE3A-A0B5-47E7-85B2-8426FB75A7C8}" name="Table_SourceData_Dairy_CropProdSystems" displayName="Table_SourceData_Dairy_CropProdSystems" ref="G7:G9" totalsRowShown="0">
+  <autoFilter ref="G7:G9" xr:uid="{B6F3FE3A-A0B5-47E7-85B2-8426FB75A7C8}">
+    <filterColumn colId="0" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{488F257E-D7D8-4266-96A1-1EA0C5DDDD42}" name="Production system">
+      <calculatedColumnFormula>#REF!</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{97BE32D2-DBFC-4EB1-B877-3886BDB57DB6}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9437,21 +9472,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B6F3FE3A-A0B5-47E7-85B2-8426FB75A7C8}" name="Table_SourceData_Dairy_CropProdSystems" displayName="Table_SourceData_Dairy_CropProdSystems" ref="G7:G9" totalsRowShown="0">
-  <autoFilter ref="G7:G9" xr:uid="{B6F3FE3A-A0B5-47E7-85B2-8426FB75A7C8}">
-    <filterColumn colId="0" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{488F257E-D7D8-4266-96A1-1EA0C5DDDD42}" name="Production system">
-      <calculatedColumnFormula>#REF!</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{4F8E62AC-6664-4F53-A138-BFDA993BA9CF}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9475,49 +9496,49 @@
     <tableColumn id="1" xr3:uid="{DC8B046E-693F-416E-B23F-18FC27E32B50}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0A3EAA01-F25D-462D-BA96-B7B4CB99562B}" name="MAT" totalsRowDxfId="79" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{0A3EAA01-F25D-462D-BA96-B7B4CB99562B}" name="MAT" totalsRowDxfId="42" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B6FC491B-0FE8-4BBC-BF8E-08B7115A1785}" name="MAP" totalsRowDxfId="78" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{B6FC491B-0FE8-4BBC-BF8E-08B7115A1785}" name="MAP" totalsRowDxfId="41" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{55883A40-C0BD-4C57-895A-A14078783B88}" name="Frost days per year" totalsRowDxfId="77" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{55883A40-C0BD-4C57-895A-A14078783B88}" name="Frost days per year" totalsRowDxfId="40" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{011EA866-D209-4A30-A492-5E6921CAAA8F}" name="Elevation" totalsRowDxfId="76" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{011EA866-D209-4A30-A492-5E6921CAAA8F}" name="Elevation" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{DC54C7D6-0D3C-4697-80C3-BEEA9B95C2A8}" name="MAP:PET" totalsRowDxfId="75" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{DC54C7D6-0D3C-4697-80C3-BEEA9B95C2A8}" name="MAP:PET" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{33B35725-0031-4EF7-9C0B-55FF30B8EAD5}" name="Min temp" totalsRowDxfId="74" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{33B35725-0031-4EF7-9C0B-55FF30B8EAD5}" name="Min temp" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{43940297-5590-44FC-A72E-FD441D3FC47D}" name="Max temp" totalsRowDxfId="73" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{43940297-5590-44FC-A72E-FD441D3FC47D}" name="Max temp" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{40E68101-FE4C-49DE-83C0-C158E308997A}" name="Min rainfall" totalsRowDxfId="72" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{40E68101-FE4C-49DE-83C0-C158E308997A}" name="Min rainfall" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A1785251-973E-4CC5-85DE-101A7D3F49E8}" name="Max rainfall" totalsRowDxfId="71" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{A1785251-973E-4CC5-85DE-101A7D3F49E8}" name="Max rainfall" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{C66FB744-44E4-4ADC-A9DC-7233E32E9FD3}" name="Min frost days" totalsRowDxfId="70" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{C66FB744-44E4-4ADC-A9DC-7233E32E9FD3}" name="Min frost days" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{84608646-367C-44FD-8B52-10DBADA161B3}" name="Max frost days" totalsRowDxfId="69" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{84608646-367C-44FD-8B52-10DBADA161B3}" name="Max frost days" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{6E9B45E6-618E-4B75-8D6C-8F6E6380947A}" name="Min elevation" totalsRowDxfId="68" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{6E9B45E6-618E-4B75-8D6C-8F6E6380947A}" name="Min elevation" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{EFF744E0-E24F-48DA-8B4D-3B2F3129E476}" name="Max elevation" totalsRowDxfId="67" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{EFF744E0-E24F-48DA-8B4D-3B2F3129E476}" name="Max elevation" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{0EAA36C3-CD55-4BE8-8379-3B3977C75B6E}" name="Min MAP:PET" totalsRowDxfId="66" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{0EAA36C3-CD55-4BE8-8379-3B3977C75B6E}" name="Min MAP:PET" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{FC138699-C5B8-43F7-907F-E1D3308E2973}" name="Max MAP:PET" totalsRowDxfId="65" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{FC138699-C5B8-43F7-907F-E1D3308E2973}" name="Max MAP:PET" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9525,7 +9546,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{EF2393AD-CFB6-4066-B4A7-363349742A80}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9535,7 +9556,7 @@
     <tableColumn id="1" xr3:uid="{06CF662C-A5E5-4DEC-9239-4CB002C0E0A2}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{CD6943B3-B254-4069-8F97-5CBFC91888FF}" name="Wet or Dry Zone" totalsRowDxfId="64" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{CD6943B3-B254-4069-8F97-5CBFC91888FF}" name="Wet or Dry Zone" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9543,7 +9564,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{F22C37E1-85CC-4916-880E-08FDCFFFE2F2}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9569,7 +9590,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{660D54FD-2935-4ECD-811D-1B2640E5CE5E}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9595,7 +9616,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{C6D91556-6041-4D39-859B-496ABDBC50F6}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
   <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9613,7 +9634,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{A7DBD304-C923-4767-94AA-F5392A218685}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
   <autoFilter ref="D153:E158" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9631,7 +9652,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{2346920B-7594-41BD-B864-BC0787F80039}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9641,7 +9662,7 @@
     <tableColumn id="1" xr3:uid="{A509C156-2300-4F59-ACB2-A4595093A2EA}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{9336E485-6CCE-4ED5-BB4F-2A0B4FB17FAC}" name="FracWET" dataDxfId="63">
+    <tableColumn id="2" xr3:uid="{9336E485-6CCE-4ED5-BB4F-2A0B4FB17FAC}" name="FracWET" dataDxfId="26">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9649,7 +9670,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{DE5BB734-49E5-4C93-8FCB-7FBE3A2C3E36}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
   <autoFilter ref="D186:H199" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9679,7 +9700,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{487CFC8F-DBEC-4AC7-AF47-6CB213F53AE7}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9689,26 +9710,8 @@
     <tableColumn id="1" xr3:uid="{9164AA51-A5A1-4E5D-92FE-56AFDF2289A9}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{AEC42C36-F3E4-47D0-8120-D6616131AD6D}" name="FracWET" dataDxfId="62" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{AEC42C36-F3E4-47D0-8120-D6616131AD6D}" name="FracWET" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{710DBAA8-85CF-4B2D-9C24-908BF4E6AD2B}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
-  <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{322BE605-15DD-4029-9C40-CCFCF7837208}" name="Climate zone">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{343D9844-A9CD-45FD-8FC0-537592119D97}" name="EFPRP" dataDxfId="61" dataCellStyle="Content normal">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -9728,6 +9731,24 @@
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{710DBAA8-85CF-4B2D-9C24-908BF4E6AD2B}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
+  <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{322BE605-15DD-4029-9C40-CCFCF7837208}" name="Climate zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{343D9844-A9CD-45FD-8FC0-537592119D97}" name="EFPRP" dataDxfId="24" dataCellStyle="Content normal">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="45" xr:uid="{58365E56-91AB-44EA-9051-27318E00FC3D}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
   <autoFilter ref="D212:E224" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9737,7 +9758,7 @@
     <tableColumn id="1" xr3:uid="{62E97CC9-F1D6-46EA-B114-90C0CA45EFBE}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DAA011C6-D7B3-4F13-B4E8-E15F8912E722}" name="Season" dataDxfId="60" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{DAA011C6-D7B3-4F13-B4E8-E15F8912E722}" name="Season" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9745,7 +9766,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="46" xr:uid="{D0584D3C-48A0-4398-9842-C522CDAA02E4}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
   <autoFilter ref="D231:S250" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9769,49 +9790,49 @@
     <tableColumn id="1" xr3:uid="{2A3DC107-6C47-44FF-87B5-2A6CE13D280F}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{65DB6E98-694B-45AA-8937-DB55FA0D8C26}" name="MAT (ºC)" dataDxfId="59" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{65DB6E98-694B-45AA-8937-DB55FA0D8C26}" name="MAT (ºC)" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{423B4300-11F0-471F-A585-18582E7C075A}" name="Anaerobic lagoon" dataDxfId="58" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{423B4300-11F0-471F-A585-18582E7C075A}" name="Anaerobic lagoon" dataDxfId="21" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{4D37A7AE-8B67-4DF0-8763-6CDE3799ABDF}" name="Digester / covered lagoons" dataDxfId="57" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{4D37A7AE-8B67-4DF0-8763-6CDE3799ABDF}" name="Digester / covered lagoons" dataDxfId="20" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DA13DDCF-E05B-49C3-96FA-E3F92DEE0475}" name="Liquid systems" dataDxfId="56" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{DA13DDCF-E05B-49C3-96FA-E3F92DEE0475}" name="Liquid systems" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{553893EA-BFAF-490D-B54B-41BF3A793E7B}" name="Daily spread" dataDxfId="55" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{553893EA-BFAF-490D-B54B-41BF3A793E7B}" name="Daily spread" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{38720A28-3C54-4788-BB84-5E69FBC36345}" name="Composting (passive windrow)" dataDxfId="54" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{38720A28-3C54-4788-BB84-5E69FBC36345}" name="Composting (passive windrow)" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{DE6E27AC-E1C2-4E80-A548-CD093BDA9B78}" name="Solid storage" dataDxfId="53" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{DE6E27AC-E1C2-4E80-A548-CD093BDA9B78}" name="Solid storage" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A8F41DBC-E4D2-4E3F-89DB-C52552BE0EC6}" name="Pit storage" dataDxfId="52" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{A8F41DBC-E4D2-4E3F-89DB-C52552BE0EC6}" name="Pit storage" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{25CAC5CA-114C-41BD-8823-6E3FAC002C2E}" name="Deep litter" dataDxfId="51" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{25CAC5CA-114C-41BD-8823-6E3FAC002C2E}" name="Deep litter" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{8268B7D2-9F2D-4085-8E81-2A4FD1305075}" name="Poultry manure with bedding" dataDxfId="50" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{8268B7D2-9F2D-4085-8E81-2A4FD1305075}" name="Poultry manure with bedding" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D7FBD043-3166-4056-B6F3-33E8243C87CD}" name="Poultry manure without bedding" dataDxfId="49" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{D7FBD043-3166-4056-B6F3-33E8243C87CD}" name="Poultry manure without bedding" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{D490DB9D-9A0D-4BB2-9724-A41FEF1E07A7}" name="Direct processing" dataDxfId="48" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{D490DB9D-9A0D-4BB2-9724-A41FEF1E07A7}" name="Direct processing" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{9B743123-9DAA-41E6-8BA4-D1A05B9012F4}" name="Direct application" dataDxfId="47" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{9B743123-9DAA-41E6-8BA4-D1A05B9012F4}" name="Direct application" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{A7DEBA54-0143-49E3-9737-BD54213DC226}" name="Pasture range and paddock" dataDxfId="46" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{A7DEBA54-0143-49E3-9737-BD54213DC226}" name="Pasture range and paddock" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{797B7FB5-A4ED-4A69-9F08-E1144CB16E77}" name="MAT raw" dataDxfId="45" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{797B7FB5-A4ED-4A69-9F08-E1144CB16E77}" name="MAT raw" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9819,7 +9840,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="49" xr:uid="{53E91874-AD42-4480-BA75-1A2818937C72}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
   <autoFilter ref="D257:E259" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -9829,7 +9850,7 @@
     <tableColumn id="1" xr3:uid="{159A749F-9D6F-43F5-8F32-7928E25410FD}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5B26F9A9-A25D-42FE-801E-E28EAB2A428B}" name="EFNi &amp; EFN2Oi" dataDxfId="44" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{5B26F9A9-A25D-42FE-801E-E28EAB2A428B}" name="EFNi &amp; EFN2Oi" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9837,9 +9858,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{757CC28B-CF78-4195-86CA-5AEBBA7FA04E}" name="Table_Data_MMSSymbols" displayName="Table_Data_MMSSymbols" ref="D8:F26" totalsRowShown="0">
-  <autoFilter ref="D8:F26" xr:uid="{757CC28B-CF78-4195-86CA-5AEBBA7FA04E}">
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{757CC28B-CF78-4195-86CA-5AEBBA7FA04E}" name="Table_Data_MMSSymbols" displayName="Table_Data_MMSSymbols" ref="D9:F27" totalsRowShown="0">
+  <autoFilter ref="D9:F27" xr:uid="{757CC28B-CF78-4195-86CA-5AEBBA7FA04E}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -9871,13 +9892,13 @@
     <tableColumn id="1" xr3:uid="{CAC4C566-E7DF-44B3-BDB4-4B1785D5F9F0}" name="Breed">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightCowsAndHeifers_Data(), Table_SourceData_Dairy_WjCowsHeifers[[#Headers],[Breed]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4C5541D8-40C3-436A-815B-7A3D9D154BB6}" name="Milking cows" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{4C5541D8-40C3-436A-815B-7A3D9D154BB6}" name="Milking cows" dataDxfId="78" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightCowsAndHeifers_Data(), Table_SourceData_Dairy_WjCowsHeifers[[#Headers],[Breed]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A8A468F3-E260-4E60-AC14-8F50FD33B46B}" name="Heifers &gt; 1" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{A8A468F3-E260-4E60-AC14-8F50FD33B46B}" name="Heifers &gt; 1" dataDxfId="77" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightCowsAndHeifers_Data(), Table_SourceData_Dairy_WjCowsHeifers[[#Headers],[Breed]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2081FE2E-69DF-48BF-9561-91AC655332BC}" name="Heifers &lt; 1 (weaned)" dataDxfId="40" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{2081FE2E-69DF-48BF-9561-91AC655332BC}" name="Heifers &lt; 1 (weaned)" dataDxfId="76" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightCowsAndHeifers_Data(), Table_SourceData_Dairy_WjCowsHeifers[[#Headers],[Breed]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9896,10 +9917,10 @@
     <tableColumn id="1" xr3:uid="{40374F5E-9BC3-4080-A28F-8B1F65DE1774}" name="Breed">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightBulls_Data(), Table_SourceData_Dairy_WjBulls[[#Headers],[Breed]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C20ABB8A-524B-457C-86CD-D1ADCBCD6339}" name="Bulls &gt; 1" dataDxfId="39" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{C20ABB8A-524B-457C-86CD-D1ADCBCD6339}" name="Bulls &gt; 1" dataDxfId="75" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightBulls_Data(), Table_SourceData_Dairy_WjBulls[[#Headers],[Breed]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{7E843FE2-40FC-4270-88C9-9204E6D4AFBC}" name="Bulls &lt; 1 (weaned)" dataDxfId="38" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{7E843FE2-40FC-4270-88C9-9204E6D4AFBC}" name="Bulls &lt; 1 (weaned)" dataDxfId="74" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightBulls_Data(), Table_SourceData_Dairy_WjBulls[[#Headers],[Breed]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9920,16 +9941,16 @@
     <tableColumn id="1" xr3:uid="{69C0AC05-6C13-494A-8124-C36C4B6D01B6}" name="Milking cows">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightGain_Data(), Table_SourceData_Dairy_LWGj[[#Headers],[Milking cows]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6F9B3B56-C4EB-4BB7-8805-05635494D786}" name="Heifers &gt; 1" dataDxfId="37" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6F9B3B56-C4EB-4BB7-8805-05635494D786}" name="Heifers &gt; 1" dataDxfId="73" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightGain_Data(), Table_SourceData_Dairy_LWGj[[#Headers],[Milking cows]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9CCB5E7F-697E-47C8-A2FC-07B0CCA18EF6}" name="Heifers &lt; 1 (weaned)" dataDxfId="36" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{9CCB5E7F-697E-47C8-A2FC-07B0CCA18EF6}" name="Heifers &lt; 1 (weaned)" dataDxfId="72" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightGain_Data(), Table_SourceData_Dairy_LWGj[[#Headers],[Milking cows]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E2F3229F-1A83-4902-9C97-123E692B43D6}" name="Bulls &gt; 1" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{E2F3229F-1A83-4902-9C97-123E692B43D6}" name="Bulls &gt; 1" dataDxfId="71" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightGain_Data(), Table_SourceData_Dairy_LWGj[[#Headers],[Milking cows]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{409BDD9D-D084-43BF-B34D-A29B0DFF00E7}" name="Bulls &lt; 1 (weaned)" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{409BDD9D-D084-43BF-B34D-A29B0DFF00E7}" name="Bulls &lt; 1 (weaned)" dataDxfId="70" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_LiveweightGain_Data(), Table_SourceData_Dairy_LWGj[[#Headers],[Milking cows]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9938,7 +9959,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{296C6784-8B86-412A-92D3-E911DE28757C}" name="Table_SourceData_Dairy_WRj" displayName="Table_SourceData_Dairy_WRj" ref="D54:H55" totalsRowShown="0" headerRowDxfId="33" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{296C6784-8B86-412A-92D3-E911DE28757C}" name="Table_SourceData_Dairy_WRj" displayName="Table_SourceData_Dairy_WRj" ref="D54:H55" totalsRowShown="0" headerRowDxfId="69" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="D54:H55" xr:uid="{296C6784-8B86-412A-92D3-E911DE28757C}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -9968,7 +9989,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{968BB314-DB2C-4CA2-BAA9-E66557777E59}" name="Table_SourceData_Dairy_DataPreWeaned" displayName="Table_SourceData_Dairy_DataPreWeaned" ref="D62:G64" totalsRowShown="0" dataDxfId="32" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{968BB314-DB2C-4CA2-BAA9-E66557777E59}" name="Table_SourceData_Dairy_DataPreWeaned" displayName="Table_SourceData_Dairy_DataPreWeaned" ref="D62:G64" totalsRowShown="0" dataDxfId="68" dataCellStyle="Content normal">
   <autoFilter ref="D62:G64" xr:uid="{968BB314-DB2C-4CA2-BAA9-E66557777E59}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -9976,16 +9997,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{598A8529-B449-4014-BE34-ECB667ED42D5}" name="Animal class j" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{598A8529-B449-4014-BE34-ECB667ED42D5}" name="Animal class j" dataDxfId="67" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_PreWeanedCalves_Data(), Table_SourceData_Dairy_DataPreWeaned[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5C0E8AAB-9E7B-4D2E-B948-D2A0CC665284}" name="CH4 production" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{5C0E8AAB-9E7B-4D2E-B948-D2A0CC665284}" name="CH4 production" dataDxfId="66" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_PreWeanedCalves_Data(), Table_SourceData_Dairy_DataPreWeaned[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{945A18DE-556C-4BC4-A6F6-B0601941462E}" name="Volatile solids (VSj=3,5)" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{945A18DE-556C-4BC4-A6F6-B0601941462E}" name="Volatile solids (VSj=3,5)" dataDxfId="65" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_PreWeanedCalves_Data(), Table_SourceData_Dairy_DataPreWeaned[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8FC08B28-B758-4413-861D-9585CC484979}" name="Nitrogen Excreted (NPWj=3,5)" dataDxfId="28" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{8FC08B28-B758-4413-861D-9585CC484979}" name="Nitrogen Excreted (NPWj=3,5)" dataDxfId="64" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_PreWeanedCalves_Data(), Table_SourceData_Dairy_DataPreWeaned[[#Headers],[Animal class j]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -10011,31 +10032,31 @@
     <tableColumn id="1" xr3:uid="{A54F6170-CD83-454D-874A-2A78490F2BD1}" name="MMS m">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B29E40EC-DE00-4962-8467-1C7A786C3DE4}" name="ACT" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B29E40EC-DE00-4962-8467-1C7A786C3DE4}" name="ACT" dataDxfId="63" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{1ABF48E7-6948-4398-A069-F461406208B9}" name="NSW" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{1ABF48E7-6948-4398-A069-F461406208B9}" name="NSW" dataDxfId="62" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A3DDB858-97C5-4EC8-955B-D48536431CC8}" name="NT" dataDxfId="25" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{A3DDB858-97C5-4EC8-955B-D48536431CC8}" name="NT" dataDxfId="61" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{64B146B6-1E4C-4E4E-A22B-B3F33B7F2C8D}" name="QLD" dataDxfId="24" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{64B146B6-1E4C-4E4E-A22B-B3F33B7F2C8D}" name="QLD" dataDxfId="60" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4AC061FD-3D5D-4347-80B4-437EEDDA407C}" name="SA" dataDxfId="23" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{4AC061FD-3D5D-4347-80B4-437EEDDA407C}" name="SA" dataDxfId="59" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{58DE1EF2-ABA1-4507-A5A2-10DBB72C5360}" name="TAS" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{58DE1EF2-ABA1-4507-A5A2-10DBB72C5360}" name="TAS" dataDxfId="58" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BA557B69-47EC-4B41-B9CC-12F16489EFF2}" name="VIC" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{BA557B69-47EC-4B41-B9CC-12F16489EFF2}" name="VIC" dataDxfId="57" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{1830500E-FEC6-4240-A1B1-EB7C6052507D}" name="WA" dataDxfId="20" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{1830500E-FEC6-4240-A1B1-EB7C6052507D}" name="WA" dataDxfId="56" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{32D3BCE1-C338-4B12-B792-DFD9C2DF0EAC}" name="NIR reference" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{32D3BCE1-C338-4B12-B792-DFD9C2DF0EAC}" name="NIR reference" dataDxfId="55" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Dairy.SourceData_Dairy_MCF_Data(), Table_SourceData_Dairy_MCFjm[[#Headers],[MMS m]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -18228,9 +18249,15 @@
       <c r="J5" s="6" t="s">
         <v>115</v>
       </c>
+      <c r="L5" s="6" t="s">
+        <v>251</v>
+      </c>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L6" s="1" t="s">
+        <v>252</v>
+      </c>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -18246,6 +18273,9 @@
       <c r="J7" s="38" t="s">
         <v>112</v>
       </c>
+      <c r="L7" s="38" t="s">
+        <v>253</v>
+      </c>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -18253,11 +18283,11 @@
         <v>0</v>
       </c>
       <c r="D8" s="38" t="str">
-        <f>'Constants - Livestock'!$E$9</f>
+        <f>'Constants - Common Livestock'!$E$10</f>
         <v>Anaerobic lagoon</v>
       </c>
       <c r="E8" s="38" t="str">
-        <f>'Constants - Livestock'!$F$9</f>
+        <f>'Constants - Common Livestock'!$F$10</f>
         <v>Anaerobic lagoon (m=1)</v>
       </c>
       <c r="G8" s="38" t="str">
@@ -18266,6 +18296,9 @@
       </c>
       <c r="J8" s="38" t="s">
         <v>116</v>
+      </c>
+      <c r="L8" s="38" t="s">
+        <v>127</v>
       </c>
       <c r="M8" s="1"/>
     </row>
@@ -18275,11 +18308,11 @@
         <v>Site</v>
       </c>
       <c r="D9" s="38" t="str">
-        <f>'Constants - Livestock'!$E$12</f>
+        <f>'Constants - Common Livestock'!$E$13</f>
         <v>Sump and dispersal system</v>
       </c>
       <c r="E9" s="38" t="str">
-        <f>'Constants - Livestock'!$F$12</f>
+        <f>'Constants - Common Livestock'!$F$13</f>
         <v>Sump and dispersal system (m=3a)</v>
       </c>
       <c r="G9" s="1" t="str">
@@ -18288,6 +18321,9 @@
       </c>
       <c r="J9" s="38" t="s">
         <v>117</v>
+      </c>
+      <c r="L9" s="38" t="s">
+        <v>144</v>
       </c>
       <c r="M9" s="1"/>
     </row>
@@ -18297,35 +18333,44 @@
         <v>Dairy</v>
       </c>
       <c r="D10" s="38" t="str">
-        <f>'Constants - Livestock'!$E$13</f>
+        <f>'Constants - Common Livestock'!$E$14</f>
         <v>Drains to paddock</v>
       </c>
       <c r="E10" s="38" t="str">
-        <f>'Constants - Livestock'!$F$13</f>
+        <f>'Constants - Common Livestock'!$F$14</f>
         <v>Drains to paddock (m=3b)</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>118</v>
       </c>
+      <c r="L10" s="38" t="s">
+        <v>145</v>
+      </c>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D11" s="38" t="str">
-        <f>'Constants - Livestock'!$E$14</f>
+        <f>'Constants - Common Livestock'!$E$15</f>
         <v>Solid storage</v>
       </c>
       <c r="E11" s="38" t="str">
-        <f>'Constants - Livestock'!$F$14</f>
+        <f>'Constants - Common Livestock'!$F$15</f>
         <v>Solid storage (m=4)</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>119</v>
+      </c>
+      <c r="L11" s="38" t="s">
+        <v>146</v>
       </c>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="J12" s="1" t="s">
         <v>120</v>
+      </c>
+      <c r="L12" s="38" t="s">
+        <v>147</v>
       </c>
       <c r="M12" s="1"/>
     </row>
@@ -20594,7 +20639,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="15">
+  <tableParts count="16">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
@@ -20610,6 +20655,7 @@
     <tablePart r:id="rId13"/>
     <tablePart r:id="rId14"/>
     <tablePart r:id="rId15"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
@@ -24856,18 +24902,12 @@
         <f>HYPERLINK("#'Results'!A1", "Results")</f>
         <v>Results</v>
       </c>
-      <c r="D5" s="6" t="str" cm="1">
-        <f t="array" ref="D5">CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Title()</f>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D6" s="6" t="str" cm="1">
+        <f t="array" ref="D6">CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Title()</f>
         <v>Table 5.12 Additional symbols used in algorithms for manure related emissions</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-    </row>
-    <row r="6" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="str" cm="1">
-        <f t="array" ref="D6">CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Vairable()</f>
-        <v>MMS</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -24875,9 +24915,9 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7" s="5" t="str" cm="1">
-        <f t="array" ref="D7">CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Source()</f>
-        <v>National Inventory Report 2023 Volume 1: Table 5.12</v>
+      <c r="D7" s="3" t="str" cm="1">
+        <f t="array" ref="D7">CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Vairable()</f>
+        <v>MMS</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -24888,15 +24928,12 @@
       <c r="A8" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>75</v>
-      </c>
+      <c r="D8" s="5" t="str" cm="1">
+        <f t="array" ref="D8">CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Source()</f>
+        <v>National Inventory Report 2023 Volume 1: Table 5.12</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
@@ -24905,17 +24942,14 @@
         <f>HYPERLINK("#'Input - Site'!A1", "Site")</f>
         <v>Site</v>
       </c>
-      <c r="D9" s="37" t="str" cm="1">
-        <f t="array" ref="D9">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>1</v>
-      </c>
-      <c r="E9" s="37" t="str" cm="1">
-        <f t="array" ref="E9">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Anaerobic lagoon</v>
-      </c>
-      <c r="F9" s="37" t="str" cm="1">
-        <f t="array" ref="F9">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Anaerobic lagoon (m=1)</v>
+      <c r="D9" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="38" t="s">
+        <v>75</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -24926,45 +24960,45 @@
       </c>
       <c r="D10" s="37" t="str" cm="1">
         <f t="array" ref="D10">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="37" t="str" cm="1">
         <f t="array" ref="E10">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Liquid systems</v>
+        <v>Anaerobic lagoon</v>
       </c>
       <c r="F10" s="37" t="str" cm="1">
         <f t="array" ref="F10">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
+        <v>Anaerobic lagoon (m=1)</v>
+      </c>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="37" t="str" cm="1">
+        <f t="array" ref="D11">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
+        <v>2</v>
+      </c>
+      <c r="E11" s="37" t="str" cm="1">
+        <f t="array" ref="E11">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
+        <v>Liquid systems</v>
+      </c>
+      <c r="F11" s="37" t="str" cm="1">
+        <f t="array" ref="F11">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
         <v>Liquid systems (m=2)</v>
-      </c>
-      <c r="G10" s="3"/>
-    </row>
-    <row r="11" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D11" s="38" t="str" cm="1">
-        <f t="array" ref="D11">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>3</v>
-      </c>
-      <c r="E11" s="38" t="str" cm="1">
-        <f t="array" ref="E11">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Daily spread</v>
-      </c>
-      <c r="F11" s="38" t="str" cm="1">
-        <f t="array" ref="F11">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Daily spread (m=3)</v>
       </c>
       <c r="G11" s="3"/>
     </row>
     <row r="12" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D12" s="38" t="str" cm="1">
         <f t="array" ref="D12">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>3a</v>
+        <v>3</v>
       </c>
       <c r="E12" s="38" t="str" cm="1">
         <f t="array" ref="E12">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Sump and dispersal system</v>
+        <v>Daily spread</v>
       </c>
       <c r="F12" s="38" t="str" cm="1">
         <f t="array" ref="F12">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Sump and dispersal system (m=3a)</v>
+        <v>Daily spread (m=3)</v>
       </c>
       <c r="G12" s="3"/>
     </row>
@@ -24974,15 +25008,15 @@
       </c>
       <c r="D13" s="38" t="str" cm="1">
         <f t="array" ref="D13">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>3b</v>
+        <v>3a</v>
       </c>
       <c r="E13" s="38" t="str" cm="1">
         <f t="array" ref="E13">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Drains to paddock</v>
+        <v>Sump and dispersal system</v>
       </c>
       <c r="F13" s="38" t="str" cm="1">
         <f t="array" ref="F13">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Drains to paddock (m=3b)</v>
+        <v>Sump and dispersal system (m=3a)</v>
       </c>
       <c r="G13" s="3"/>
     </row>
@@ -24993,45 +25027,45 @@
       </c>
       <c r="D14" s="38" t="str" cm="1">
         <f t="array" ref="D14">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>4</v>
+        <v>3b</v>
       </c>
       <c r="E14" s="38" t="str" cm="1">
         <f t="array" ref="E14">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Solid storage</v>
+        <v>Drains to paddock</v>
       </c>
       <c r="F14" s="38" t="str" cm="1">
         <f t="array" ref="F14">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Solid storage (m=4)</v>
+        <v>Drains to paddock (m=3b)</v>
       </c>
       <c r="G14" s="3"/>
     </row>
     <row r="15" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D15" s="38" t="str" cm="1">
         <f t="array" ref="D15">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="38" t="str" cm="1">
         <f t="array" ref="E15">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Drylot (feed pad)</v>
+        <v>Solid storage</v>
       </c>
       <c r="F15" s="38" t="str" cm="1">
         <f t="array" ref="F15">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Drylot (feed pad) (m=5)</v>
+        <v>Solid storage (m=4)</v>
       </c>
       <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D16" s="38" t="str" cm="1">
         <f t="array" ref="D16">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="38" t="str" cm="1">
         <f t="array" ref="E16">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Composting (passive windrow)</v>
+        <v>Drylot (feed pad)</v>
       </c>
       <c r="F16" s="38" t="str" cm="1">
         <f t="array" ref="F16">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Composting (passive windrow) (m=6)</v>
+        <v>Drylot (feed pad) (m=5)</v>
       </c>
       <c r="G16" s="3"/>
     </row>
@@ -25041,15 +25075,15 @@
       </c>
       <c r="D17" s="38" t="str" cm="1">
         <f t="array" ref="D17">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="38" t="str" cm="1">
         <f t="array" ref="E17">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Digester / covered lagoons</v>
+        <v>Composting (passive windrow)</v>
       </c>
       <c r="F17" s="38" t="str" cm="1">
         <f t="array" ref="F17">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Digester / covered lagoons (m=7)</v>
+        <v>Composting (passive windrow) (m=6)</v>
       </c>
       <c r="G17" s="3"/>
     </row>
@@ -25060,15 +25094,15 @@
       </c>
       <c r="D18" s="38" t="str" cm="1">
         <f t="array" ref="D18">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="38" t="str" cm="1">
         <f t="array" ref="E18">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Deep litter</v>
+        <v>Digester / covered lagoons</v>
       </c>
       <c r="F18" s="38" t="str" cm="1">
         <f t="array" ref="F18">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Deep litter (m=8)</v>
+        <v>Digester / covered lagoons (m=7)</v>
       </c>
       <c r="G18" s="3"/>
     </row>
@@ -25079,15 +25113,15 @@
       </c>
       <c r="D19" s="38" t="str" cm="1">
         <f t="array" ref="D19">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="38" t="str" cm="1">
         <f t="array" ref="E19">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Pit storage</v>
+        <v>Deep litter</v>
       </c>
       <c r="F19" s="38" t="str" cm="1">
         <f t="array" ref="F19">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Pit storage (m=9)</v>
+        <v>Deep litter (m=8)</v>
       </c>
       <c r="G19" s="3"/>
     </row>
@@ -25098,15 +25132,15 @@
       </c>
       <c r="D20" s="38" t="str" cm="1">
         <f t="array" ref="D20">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E20" s="38" t="str" cm="1">
         <f t="array" ref="E20">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Poultry manure with bedding</v>
+        <v>Pit storage</v>
       </c>
       <c r="F20" s="38" t="str" cm="1">
         <f t="array" ref="F20">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Poultry manure with bedding (m=10)</v>
+        <v>Pit storage (m=9)</v>
       </c>
       <c r="G20" s="3"/>
     </row>
@@ -25117,94 +25151,107 @@
       </c>
       <c r="D21" s="38" t="str" cm="1">
         <f t="array" ref="D21">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E21" s="38" t="str" cm="1">
         <f t="array" ref="E21">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Poultry manure without bedding</v>
+        <v>Poultry manure with bedding</v>
       </c>
       <c r="F21" s="38" t="str" cm="1">
         <f t="array" ref="F21">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Poultry manure without bedding (m=11)</v>
+        <v>Poultry manure with bedding (m=10)</v>
       </c>
       <c r="G21" s="3"/>
     </row>
     <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D22" s="38" t="str" cm="1">
         <f t="array" ref="D22">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>11a</v>
+        <v>11</v>
       </c>
       <c r="E22" s="38" t="str" cm="1">
         <f t="array" ref="E22">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Belt manure removal</v>
+        <v>Poultry manure without bedding</v>
       </c>
       <c r="F22" s="38" t="str" cm="1">
         <f t="array" ref="F22">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Belt manure removal (m=11a)</v>
+        <v>Poultry manure without bedding (m=11)</v>
       </c>
       <c r="G22" s="3"/>
     </row>
     <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D23" s="38" t="str" cm="1">
         <f t="array" ref="D23">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>11b</v>
+        <v>11a</v>
       </c>
       <c r="E23" s="38" t="str" cm="1">
         <f t="array" ref="E23">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Manure stored in house</v>
+        <v>Belt manure removal</v>
       </c>
       <c r="F23" s="38" t="str" cm="1">
         <f t="array" ref="F23">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Manure stored in house (m=11b)</v>
+        <v>Belt manure removal (m=11a)</v>
       </c>
       <c r="G23" s="3"/>
     </row>
     <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D24" s="38" t="str" cm="1">
         <f t="array" ref="D24">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>12</v>
+        <v>11b</v>
       </c>
       <c r="E24" s="38" t="str" cm="1">
         <f t="array" ref="E24">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Direct processing</v>
+        <v>Manure stored in house</v>
       </c>
       <c r="F24" s="38" t="str" cm="1">
         <f t="array" ref="F24">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Direct processing (m=12)</v>
+        <v>Manure stored in house (m=11b)</v>
       </c>
       <c r="G24" s="3"/>
     </row>
     <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" s="38" t="str" cm="1">
         <f t="array" ref="D25">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E25" s="38" t="str" cm="1">
         <f t="array" ref="E25">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Direct application</v>
+        <v>Direct processing</v>
       </c>
       <c r="F25" s="38" t="str" cm="1">
         <f t="array" ref="F25">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Direct application (m=13)</v>
+        <v>Direct processing (m=12)</v>
       </c>
       <c r="G25" s="3"/>
     </row>
     <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D26" s="38" t="str" cm="1">
         <f t="array" ref="D26">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26" s="38" t="str" cm="1">
         <f t="array" ref="E26">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
-        <v>Pasture range and paddock</v>
+        <v>Direct application</v>
       </c>
       <c r="F26" s="38" t="str" cm="1">
         <f t="array" ref="F26">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
+        <v>Direct application (m=13)</v>
+      </c>
+      <c r="G26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D27" s="38" t="str" cm="1">
+        <f t="array" ref="D27">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
+        <v>14</v>
+      </c>
+      <c r="E27" s="38" t="str" cm="1">
+        <f t="array" ref="E27">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
+        <v>Pasture range and paddock</v>
+      </c>
+      <c r="F27" s="38" t="str" cm="1">
+        <f t="array" ref="F27">Common_InputFunctions.Utility_DisplayArrayInTable(CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data(), Table_Data_MMSSymbols[[#Headers],[Symbol]], 0)</f>
         <v>Pasture range and paddock (m=14)</v>
       </c>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    </row>
     <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
@@ -25254,6 +25301,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAXAB1ADAAMAAyADcAUgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcALAAgAGEAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAaQBzACAAYwBvAG4AcwBpAHMAdABlAG4AdABsAHkAIABcAHUAMAAwADIANwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdAFwAdQAwADAAMgA3ACAAYQBuAGQAIABpAHMAIABuAG8AdAAgAHUAcwBlAGQAIABpAG4AIABjAGEAbABjAHUAbABhAHQAaQBvAG4ALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHIAZQBlAGQAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBsAGwAIABiAHIAZQBlAGQAcwBcACIALAAgADYAMAAwACwAIAAyADIANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAVwBHAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA1ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABDAG8AdwBzAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAANQA5ADAALAAgADUAOQAwACwAIAA1ADkAMAAsACAANwA3ADAALAAgADcANwAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAdABhACAAZgBvAHIAIABwAHIAZQAgAC0AIAB3AGUAYQBuAGUAZAAgAGMAYQBsAHYAZQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBqAD0AMwAsADUAOwAgAE4AUABXAGoAPQAzACwANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzAFwAdQAwADAAMwBjADEAXAAiACwAIAAwAC4AMAAxADcANgAsACAAMAAuADIANgA4ADUALAAgADAALgAwADEAMwA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwBcAHUAMAAwADMAYwAxAFwAIgAsACAAMAAuADAAMgAwADQALAAgADAALgAzADAAMAAzACwAIAAwAC4AMAAwADkAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBDAEYAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEAMAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBUAEEAUwBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAuADcAMgAsACAAMAAuADcANgAsACAAMAAuADgALAAgADAALgA3ADgALAAgADAALgA3ADQALAAgADAALgA2ADkALAAgADAALgA3ADMALAAgADAALgA3ADYALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwAgACgAYQApAFwAIgAsACAAMAAuADEANQAsACAAMAAuADEAOAAsACAAMAAuADUAMAAsACAAMAAuADIANAAsACAAMAAuADEANwAsACAAMAAuADEAMwAsACAAMAAuADEANwAsACAAMAAuADEAOAAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAG0AOwAgAEYAcgBhAGMARwBBAFMATQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADAALgAwADEANwA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjACAAMQAgAHkAZQBhAHIAXAAiACwAIAAwAC4AMAAyADAANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBSAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA5ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABJAG4AYwByAGUAYQBzAGUAZAAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAIAAoAE0AUgBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUgBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFIAagBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMALAAgAGEAbgBkACAAaABvAHUAcwBlACAAYwBvAHcAcwBcACIALAAgADEALgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAbwB0AGgAZQByACAAYwBhAHQAdABsAGUAIABjAGwAYQBzAHMAZQBzAFwAIgAsACAAMQAuADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAdgBvAGkAZABlAGQAIAB0AG8AIABlAGEAYwBoACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAE0AUwBqAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBqAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEUAeABjAGwAdQBkAGUAZAAgAFwAdQAwADAAMgA3AEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQBcAHUAMAAwADIANwAgAHIAbwB3ACAAYQBzACAAdABoAGkAcwAgAGkAbgBmAG8AcgBtAGEAdABpAG8AbgAgAGkAcwAgAGkAbgAgAHQAaABlACAAdABhAGIAbABlACAAdABpAHQAbABlAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQByAGUAYQBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE0AaQBsAGsAaQBuAGcAIABTAGgAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAcABhAGQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMQA6ACAARwByAGEAegBlAGQAIABPAG4AbAB5AFwAIgAsACAAMAAuADgAOQAsACAAMAAuADEAMQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADIAOgAgAE8AbgAgAGYAZQBlAGQAcABhAGQAIABmAG8AcgAgAFwAdQAwADAAMwBjADEAMAAgAGgAcgAvAGQAYQB5ACAAZgBvAHIAIABcAHUAMAAwADMAYwAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMwAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEANAAgAFAAYQBzAHQAdQByAGUAXAAiACwAIAAwACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEAIABBAG4AZQByAG8AYgBpAGMAIABMAGEAZwBvAG8AbgBcACIALAAgADAALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbABcACIALAAgADAALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMwAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwBcACIALAAgADAALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQA0ACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXABuAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABmAG8AcgAgAGUAYQBjAGgAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgBwAHUAdAAgAGMAbABhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGEAeQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADIAXAB0AEQAQQBUAEEAIAAoAE0ARQBUAEgATwBEACAAMQAgAEEATgBEACAAMgAgAE8AUABUAEkATwBOAFMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBlAGUAIAB0AGUAeAB0ACAAaQBuACAAZABvAGMAdQBtAGUAbgB0ACAAdABvACAAdABhAGIAbABlACwAIABtAGEAdABjAGgAaQBuAGcAIABsAGkAdgBlAHMAdABvAGMAawAgAGMAbABhAHMAcwAgAG4AYQBtAGUAcwAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEQAdQByAGEAdABpAG8AbgAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHAAcgBlAC0AdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMAXAAiACwAIAAzADYANQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAgADEAIAB5AGUAYQByAFwAIgAsACAAMgA4ADEALAAgADgANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAgADEAIAB5AGUAYQByAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBEAGUAZgBhAHUAbAB0ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAB3AGgAZQBuACAAbQBhAG4AdQByAGUAIABpAHMAIABlAHgAYwByAGUAdABlAGQAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQAuACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAZQBmAGEAdQBsAHQAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAHcAaABlAG4AIABtAGEAbgB1AHIAZQAgAGkAcwAgAGUAeABjAHIAZQB0AGUAZAAgAHQAbwAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawAgACgAbQA9ADEANAApAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAyADQAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4ARgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBDAF8AagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQALgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAFwAbgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADIAIABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAzACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcARABQAFcAXAB1ADAAMAAyADcAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABoAGEAbgBkAGwAaQBuAGcAIABvAGYAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAZAB1AHIAYQB0AGkAbwBuAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXABuAE0AXwBqAFwAbgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ASQBfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABJAF8AagAsAFwAbgAgACAAIAAgADIAMAAuADcAIAAqACAASQBfAGoAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGgAYQByAG0AbABlAHkAIABlAHQAIABhAGwALgAgACgAMgAwADEANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADMAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4ARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgBJAF8AagBcAG4AawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAbgBXAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQBcAG4ATABXAEcAXwBqACAAPQAgAGwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATQBSAF8AagAgAD0AIABpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ATQBJAF8AagAgAD0AIABhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABXAF8AagAsACAATABXAEcAXwBqACwAIABNAFIAXwBqACwAIABNAEkAXwBqACwAXABuACAAIAAgACAAKAAxAC4AMQA4ADUAIAArACAAMAAuADAAMAA0ADUANAAgACoAIABXAF8AagAgAC0AIAAwAC4AMAAwADAAMAAwADIANgAgACoAIABXAF8AagAgAF4AIAAyACAAKwAgADAALgAzADEANQAgACoAIABMAFcARwBfAGoAKQAgAF4AIAAyACAAKgAgAE0AUgBfAGoAIAArACAATQBJAF8AagBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0AFwAIgAsACAAXAAiAGsAZwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAVwBHAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgBcACIALAAgAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFIAXwBqAFwAIgAsACAAXAAiAGkAbgBjAHIAZQBhAHMAZQAgAGkAbgAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBJAF8AagBcACIALAAgAFwAIgBhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAE0ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBJAF8AagA9ACgATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFACkALwAoAEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqACkAXABuAE0AUABfAGoAIAA9ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAEwALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATgBFACAAPQAgAG4AZQB0ACAAZQBuAGUAcgBnAHkAIAAoAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrACkAXABuAEcARQBDACAAPQAgAGcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgACgATQBKAC8AawBnAEQATQApAFwAbgBrACAAPQAgAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgBxAG0AXwBqACAAPQAgAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFAAXwBqACwAIABOAEUALAAgAEcARQBDACwAIABrACwAIABxAG0AXwBqACwAXABuACAAIAAgACAAKABNAFAAXwBqACAAKgAgADEALgAwADMAIAAqACAATgBFACkAIAAvACAAKABHAEUAQwAgACoAIABrACAAKgAgAHEAbQBfAGoAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADQAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAD0AXABcAGYAcgBhAGMAewBNAFAAXwBqAFwAXAB0AGkAbQBlAHMAIAAxAC4AMAAzAFwAXAB0AGkAbQBlAHMAIABOAEUAfQB7AEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAXwBqAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABpAGYAIABpAG4AcAB1AHQAIABhAHMAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsAKQBcACIALAAgAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBFAFwAIgAsACAAXAAiAG4AZQB0ACAAZQBuAGUAcgBnAHkAXAAiACwAIABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAvAGsAZwAgAG0AaQBsAGsAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEUAQwBcACIALAAgAFwAIgBnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAXAAiACwAIABcACIATQBKAC8AawBnAEQATQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGsAXAAiACwAIABcACIAZQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAG0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUAIABlAG4AZQByAGcAeQAgAHUAcwBlACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAG0AXwBqAFwAIgAsACAAXAAiAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgANgApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAFwAbgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcAG4ATQBQAF8AagBcAG4ATAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBQAF8AagA9AE0AUwBfAGoALwAoADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQApAFwAbgBNAFMAXwBqACAAPQAgAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIAAoAGsAZwAgAE0AUwAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBGAEMAXwBqACAAPQAgAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4AUABDAF8AagAgAD0AIABwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFMAXwBqACwAIABGAEMAXwBqACwAIABQAEMAXwBqACwAXABuACAAIAAgACAATQBTAF8AagAgAC8AIAAoADAALgAwADEAIAAqACAAKABGAEMAXwBqACAAKwAgAFAAQwBfAGoAKQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAYwBvAG4AdgBlAHIAdABlAGQAIABmAHIAbwBtACAAbQBpAGwAawAgAHMAbwBsAGkAZABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagA9AFwAXABmAHIAYQBjAHsATQBTAF8AagB9AHsAMAAuADAAMQBcAFwAdABpAG0AZQBzACAAKABGAEMAXwBqACsAUABDAF8AagApAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAGkAbgBwAHUAdAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdAAgAHYAYQByAGkAYQBiAGwAZQAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAdQBzAGUAIABvAGYAIABlAGkAdABoAGUAcgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwAgAG8AcgAgAGwAaQB0AHIAZQBzACAAbwBmACAAbQBpAGwAawAuACAAQwBvAG4AdgBlAHIAdABlAGQAIABpAG4AcAB1AHQAIABGAEMAIABhAG4AZAAgAFAAQwAgAHAAZQByAGMAZQBuAHQAIAB0AG8AIABpAG4AdABlAGcAZQByAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQAgAG8AZgAgAGQAaQBlAHQAXABuAHEAbQBfAGoAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4AcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcAG4ARABNAEQAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQATQBEAF8AagAsAFwAbgAgACAAIAAgADAALgA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABNAEQAXwBqACwAXABuACAAIAAgACAAMAAuADAAMAA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBxAG0AXwBqAD0AMAAuADAAMAA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABjAGgAYQBuAGcAZQBkACAAMAAuADcAOQA1ACAAdABvACAAMAAuADAAMAA3ADkANQAgAHcAaABpAGMAaAAgAGkAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAdQBzAGUAZAAgAGkAbgAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdABcACIAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBEAGEAaQByAHkAIgAsACIAdABlAHgAdAAiADoAIgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAE0ATQBTAEEAZgB0AGUAcgBTAG8AbABpAGQAUwBlAHAAYQByAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAsACAARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAgACoAIAAoAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAtACgATQBNAFMARgByAGEAYwB0AGkAbwBuACoARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACkAKQBcAG4AKQA7AFwAbgBcAG4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAsAFwAbgAgACAAIAAgAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMgBTAGUAcABhAHIAYQB0AGUAZAAsACAAXABuACAAIAAgACAATQBNAFMAMwBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgAXABuACAAIAAgACAAIAAgACAAIABJAG4AaQB0AGEAbABTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBGAHIAYQBjAHQAaQBvAG4AIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAxAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAzAFMAZQBwAGEAcgBhAHQAZQBkACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -25448,31 +25519,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAXAB1ADAAMAAyADcAUgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcALAAgAGEAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAaQBzACAAYwBvAG4AcwBpAHMAdABlAG4AdABsAHkAIABcAHUAMAAwADIANwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdAFwAdQAwADAAMgA3ACAAYQBuAGQAIABpAHMAIABuAG8AdAAgAHUAcwBlAGQAIABpAG4AIABjAGEAbABjAHUAbABhAHQAaQBvAG4ALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHIAZQBlAGQAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBsAGwAIABiAHIAZQBlAGQAcwBcACIALAAgADYAMAAwACwAIAAyADIANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAVwBHAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA1ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABDAG8AdwBzAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAANQA5ADAALAAgADUAOQAwACwAIAA1ADkAMAAsACAANwA3ADAALAAgADcANwAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAdABhACAAZgBvAHIAIABwAHIAZQAgAC0AIAB3AGUAYQBuAGUAZAAgAGMAYQBsAHYAZQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBqAD0AMwAsADUAOwAgAE4AUABXAGoAPQAzACwANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzAFwAdQAwADAAMwBjADEAXAAiACwAIAAwAC4AMAAxADcANgAsACAAMAAuADIANgA4ADUALAAgADAALgAwADEAMwA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwBcAHUAMAAwADMAYwAxAFwAIgAsACAAMAAuADAAMgAwADQALAAgADAALgAzADAAMAAzACwAIAAwAC4AMAAwADkAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBDAEYAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEAMAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBUAEEAUwBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAuADcAMgAsACAAMAAuADcANgAsACAAMAAuADgALAAgADAALgA3ADgALAAgADAALgA3ADQALAAgADAALgA2ADkALAAgADAALgA3ADMALAAgADAALgA3ADYALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwAgACgAYQApAFwAIgAsACAAMAAuADEANQAsACAAMAAuADEAOAAsACAAMAAuADUAMAAsACAAMAAuADIANAAsACAAMAAuADEANwAsACAAMAAuADEAMwAsACAAMAAuADEANwAsACAAMAAuADEAOAAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAG0AOwAgAEYAcgBhAGMARwBBAFMATQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADAALgAwADEANwA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjACAAMQAgAHkAZQBhAHIAXAAiACwAIAAwAC4AMAAyADAANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBSAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA5ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABJAG4AYwByAGUAYQBzAGUAZAAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAIAAoAE0AUgBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUgBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFIAagBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMALAAgAGEAbgBkACAAaABvAHUAcwBlACAAYwBvAHcAcwBcACIALAAgADEALgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAbwB0AGgAZQByACAAYwBhAHQAdABsAGUAIABjAGwAYQBzAHMAZQBzAFwAIgAsACAAMQAuADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAdgBvAGkAZABlAGQAIAB0AG8AIABlAGEAYwBoACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAE0AUwBqAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBqAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEUAeABjAGwAdQBkAGUAZAAgAFwAdQAwADAAMgA3AEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQBcAHUAMAAwADIANwAgAHIAbwB3ACAAYQBzACAAdABoAGkAcwAgAGkAbgBmAG8AcgBtAGEAdABpAG8AbgAgAGkAcwAgAGkAbgAgAHQAaABlACAAdABhAGIAbABlACAAdABpAHQAbABlAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQByAGUAYQBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE0AaQBsAGsAaQBuAGcAIABTAGgAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAcABhAGQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMQA6ACAARwByAGEAegBlAGQAIABPAG4AbAB5AFwAIgAsACAAMAAuADgAOQAsACAAMAAuADEAMQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADIAOgAgAE8AbgAgAGYAZQBlAGQAcABhAGQAIABmAG8AcgAgAFwAdQAwADAAMwBjADEAMAAgAGgAcgAvAGQAYQB5ACAAZgBvAHIAIABcAHUAMAAwADMAYwAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMwAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEANAAgAFAAYQBzAHQAdQByAGUAXAAiACwAIAAwACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEAIABBAG4AZQByAG8AYgBpAGMAIABMAGEAZwBvAG8AbgBcACIALAAgADAALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbABcACIALAAgADAALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMwAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwBcACIALAAgADAALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQA0ACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXABuAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABmAG8AcgAgAGUAYQBjAGgAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgBwAHUAdAAgAGMAbABhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGEAeQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADIAXAB0AEQAQQBUAEEAIAAoAE0ARQBUAEgATwBEACAAMQAgAEEATgBEACAAMgAgAE8AUABUAEkATwBOAFMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBlAGUAIAB0AGUAeAB0ACAAaQBuACAAZABvAGMAdQBtAGUAbgB0ACAAdABvACAAdABhAGIAbABlACwAIABtAGEAdABjAGgAaQBuAGcAIABsAGkAdgBlAHMAdABvAGMAawAgAGMAbABhAHMAcwAgAG4AYQBtAGUAcwAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEQAdQByAGEAdABpAG8AbgAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHAAcgBlAC0AdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMAXAAiACwAIAAzADYANQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAgADEAIAB5AGUAYQByAFwAIgAsACAAMgA4ADEALAAgADgANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAgADEAIAB5AGUAYQByAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBEAGUAZgBhAHUAbAB0ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAB3AGgAZQBuACAAbQBhAG4AdQByAGUAIABpAHMAIABlAHgAYwByAGUAdABlAGQAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQAuACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAZQBmAGEAdQBsAHQAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAHcAaABlAG4AIABtAGEAbgB1AHIAZQAgAGkAcwAgAGUAeABjAHIAZQB0AGUAZAAgAHQAbwAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawAgACgAbQA9ADEANAApAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAyADQAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4ARgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBDAF8AagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQALgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAFwAbgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADIAIABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAzACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcARABQAFcAXAB1ADAAMAAyADcAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABoAGEAbgBkAGwAaQBuAGcAIABvAGYAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAZAB1AHIAYQB0AGkAbwBuAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXABuAE0AXwBqAFwAbgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ASQBfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABJAF8AagAsAFwAbgAgACAAIAAgADIAMAAuADcAIAAqACAASQBfAGoAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGgAYQByAG0AbABlAHkAIABlAHQAIABhAGwALgAgACgAMgAwADEANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADMAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4ARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgBJAF8AagBcAG4AawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAbgBXAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQBcAG4ATABXAEcAXwBqACAAPQAgAGwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATQBSAF8AagAgAD0AIABpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ATQBJAF8AagAgAD0AIABhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABXAF8AagAsACAATABXAEcAXwBqACwAIABNAFIAXwBqACwAIABNAEkAXwBqACwAXABuACAAIAAgACAAKAAxAC4AMQA4ADUAIAArACAAMAAuADAAMAA0ADUANAAgACoAIABXAF8AagAgAC0AIAAwAC4AMAAwADAAMAAwADIANgAgACoAIABXAF8AagAgAF4AIAAyACAAKwAgADAALgAzADEANQAgACoAIABMAFcARwBfAGoAKQAgAF4AIAAyACAAKgAgAE0AUgBfAGoAIAArACAATQBJAF8AagBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0AFwAIgAsACAAXAAiAGsAZwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAVwBHAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgBcACIALAAgAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFIAXwBqAFwAIgAsACAAXAAiAGkAbgBjAHIAZQBhAHMAZQAgAGkAbgAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBJAF8AagBcACIALAAgAFwAIgBhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAE0ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBJAF8AagA9ACgATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFACkALwAoAEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqACkAXABuAE0AUABfAGoAIAA9ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAEwALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATgBFACAAPQAgAG4AZQB0ACAAZQBuAGUAcgBnAHkAIAAoAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrACkAXABuAEcARQBDACAAPQAgAGcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgACgATQBKAC8AawBnAEQATQApAFwAbgBrACAAPQAgAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgBxAG0AXwBqACAAPQAgAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFAAXwBqACwAIABOAEUALAAgAEcARQBDACwAIABrACwAIABxAG0AXwBqACwAXABuACAAIAAgACAAKABNAFAAXwBqACAAKgAgADEALgAwADMAIAAqACAATgBFACkAIAAvACAAKABHAEUAQwAgACoAIABrACAAKgAgAHEAbQBfAGoAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADQAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAD0AXABcAGYAcgBhAGMAewBNAFAAXwBqAFwAXAB0AGkAbQBlAHMAIAAxAC4AMAAzAFwAXAB0AGkAbQBlAHMAIABOAEUAfQB7AEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAXwBqAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABpAGYAIABpAG4AcAB1AHQAIABhAHMAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsAKQBcACIALAAgAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBFAFwAIgAsACAAXAAiAG4AZQB0ACAAZQBuAGUAcgBnAHkAXAAiACwAIABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAvAGsAZwAgAG0AaQBsAGsAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEUAQwBcACIALAAgAFwAIgBnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAXAAiACwAIABcACIATQBKAC8AawBnAEQATQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGsAXAAiACwAIABcACIAZQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAG0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUAIABlAG4AZQByAGcAeQAgAHUAcwBlACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAG0AXwBqAFwAIgAsACAAXAAiAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgANgApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAFwAbgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcAG4ATQBQAF8AagBcAG4ATAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBQAF8AagA9AE0AUwBfAGoALwAoADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQApAFwAbgBNAFMAXwBqACAAPQAgAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIAAoAGsAZwAgAE0AUwAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBGAEMAXwBqACAAPQAgAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4AUABDAF8AagAgAD0AIABwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFMAXwBqACwAIABGAEMAXwBqACwAIABQAEMAXwBqACwAXABuACAAIAAgACAATQBTAF8AagAgAC8AIAAoADAALgAwADEAIAAqACAAKABGAEMAXwBqACAAKwAgAFAAQwBfAGoAKQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAYwBvAG4AdgBlAHIAdABlAGQAIABmAHIAbwBtACAAbQBpAGwAawAgAHMAbwBsAGkAZABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagA9AFwAXABmAHIAYQBjAHsATQBTAF8AagB9AHsAMAAuADAAMQBcAFwAdABpAG0AZQBzACAAKABGAEMAXwBqACsAUABDAF8AagApAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAGkAbgBwAHUAdAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdAAgAHYAYQByAGkAYQBiAGwAZQAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAdQBzAGUAIABvAGYAIABlAGkAdABoAGUAcgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwAgAG8AcgAgAGwAaQB0AHIAZQBzACAAbwBmACAAbQBpAGwAawAuACAAQwBvAG4AdgBlAHIAdABlAGQAIABpAG4AcAB1AHQAIABGAEMAIABhAG4AZAAgAFAAQwAgAHAAZQByAGMAZQBuAHQAIAB0AG8AIABpAG4AdABlAGcAZQByAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQAgAG8AZgAgAGQAaQBlAHQAXABuAHEAbQBfAGoAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4AcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcAG4ARABNAEQAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQATQBEAF8AagAsAFwAbgAgACAAIAAgADAALgA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABNAEQAXwBqACwAXABuACAAIAAgACAAMAAuADAAMAA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBxAG0AXwBqAD0AMAAuADAAMAA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABjAGgAYQBuAGcAZQBkACAAMAAuADcAOQA1ACAAdABvACAAMAAuADAAMAA3ADkANQAgAHcAaABpAGMAaAAgAGkAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAdQBzAGUAZAAgAGkAbgAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdABcACIAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBEAGEAaQByAHkAIgAsACIAdABlAHgAdAAiADoAIgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAE0ATQBTAEEAZgB0AGUAcgBTAG8AbABpAGQAUwBlAHAAYQByAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAsACAARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAgACoAIAAoAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAtACgATQBNAFMARgByAGEAYwB0AGkAbwBuACoARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACkAKQBcAG4AKQA7AFwAbgBcAG4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAsAFwAbgAgACAAIAAgAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMgBTAGUAcABhAHIAYQB0AGUAZAAsACAAXABuACAAIAAgACAATQBNAFMAMwBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgAXABuACAAIAAgACAAIAAgACAAIABJAG4AaQB0AGEAbABTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBGAHIAYQBjAHQAaQBvAG4AIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAxAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAzAFMAZQBwAGEAcgBhAHQAZQBkACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25489,31 +25563,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(enterprise): import canonical Manure module before Enteric so master input sheet owns workbook-scoped names
</commit_message>
<xml_diff>
--- a/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
+++ b/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC60738-71C9-42DB-B6BD-B0E4C16B8179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58CC47D5-92D1-45A3-A086-29884E322BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" activeTab="5" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="990" yWindow="1215" windowWidth="36255" windowHeight="19140" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -556,8 +556,8 @@
     <definedName name="VEERG_3_3_1_1__1_TotalAnnualMethaneFromEntericFermentationVariation_Result_Method1">'3.3.1.1-2 Enteric Methane'!$E$182</definedName>
     <definedName name="VEERG_3_3_1_1__1_TotalAnnualMethaneFromEntericFermentationVariation_Result_Method2">'3.3.1.1-2 Enteric Methane'!$N$182</definedName>
     <definedName name="X_Cell_Dairy_Breed">'Input - Dairy'!$E$7</definedName>
-    <definedName name="X_Cell_Dairy_MilkProductionAmount">'Input - Dairy'!$E$52</definedName>
-    <definedName name="X_Cell_Dairy_MilkProductionUnit">'Input - Dairy'!$E$49</definedName>
+    <definedName name="X_Cell_Dairy_MilkProductionAmount">'Input - Dairy'!$E$50</definedName>
+    <definedName name="X_Cell_Dairy_MilkProductionUnit">'Input - Dairy'!$E$47</definedName>
     <definedName name="X_Cell_Site_AverageTemperature">'Input - Site'!$E$25</definedName>
     <definedName name="X_Cell_Site_ClimateZone">'Input - Site'!$E$31</definedName>
     <definedName name="X_Cell_Site_Elevation">'Input - Site'!$E$24</definedName>
@@ -582,7 +582,7 @@
     <definedName name="X_Table_Dairy_HerdMovement">'Input - Dairy'!$D$9:$I$10</definedName>
     <definedName name="X_Table_Dairy_Liveweight_Method1">'Input - Dairy'!$D$13:$I$15</definedName>
     <definedName name="X_Table_Dairy_Liveweight_Method2">'Input - Dairy'!$D$17:$I$19</definedName>
-    <definedName name="X_Table_Dairy_MilkSolidAttributes">'Input - Dairy'!$D$54:$F$56</definedName>
+    <definedName name="X_Table_Dairy_MilkSolidAttributes">'Input - Dairy'!$D$52:$F$54</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -15152,38 +15152,58 @@
       <c r="R42" s="7"/>
     </row>
     <row r="43" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
       <c r="R43" s="7"/>
     </row>
     <row r="44" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C44" s="46"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="46"/>
+      <c r="I44" s="46"/>
+      <c r="J44" s="46"/>
+      <c r="K44" s="46"/>
+      <c r="L44" s="46"/>
+      <c r="M44" s="46"/>
+      <c r="N44" s="46"/>
       <c r="R44" s="7"/>
     </row>
     <row r="45" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D45" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
       <c r="R45" s="7"/>
     </row>
     <row r="46" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="46"/>
-      <c r="D46" s="46"/>
-      <c r="E46" s="46"/>
-      <c r="F46" s="46"/>
-      <c r="G46" s="46"/>
-      <c r="H46" s="46"/>
-      <c r="I46" s="46"/>
-      <c r="J46" s="46"/>
-      <c r="K46" s="46"/>
-      <c r="L46" s="46"/>
-      <c r="M46" s="46"/>
-      <c r="N46" s="46"/>
+      <c r="G46" s="6"/>
+      <c r="H46" s="6"/>
+      <c r="I46" s="6"/>
+      <c r="J46" s="113"/>
+      <c r="K46" s="113"/>
+      <c r="L46" s="113"/>
+      <c r="M46" s="113"/>
       <c r="R46" s="7"/>
     </row>
     <row r="47" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D47" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
+      <c r="D47" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="E47" s="41" t="s">
+        <v>248</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
@@ -15193,104 +15213,82 @@
       <c r="R47" s="7"/>
     </row>
     <row r="48" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="113"/>
-      <c r="K48" s="113"/>
-      <c r="L48" s="113"/>
-      <c r="M48" s="113"/>
       <c r="R48" s="7"/>
     </row>
     <row r="49" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D49" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="E49" s="41" t="s">
-        <v>248</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="3"/>
-      <c r="K49" s="3"/>
-      <c r="L49" s="3"/>
-      <c r="M49" s="3"/>
+      <c r="E49" s="40" t="s">
+        <v>127</v>
+      </c>
       <c r="R49" s="7"/>
     </row>
     <row r="50" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="R50" s="7"/>
-    </row>
-    <row r="51" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E51" s="40" t="s">
-        <v>127</v>
-      </c>
-      <c r="R51" s="7"/>
-    </row>
-    <row r="52" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D52" s="1" t="s">
+      <c r="D50" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E52" s="64">
+      <c r="E50" s="64">
         <v>20</v>
       </c>
-      <c r="F52" s="2" t="str">
+      <c r="F50" s="2" t="str">
         <f>IF(X_Cell_Dairy_MilkProductionUnit="Litres of milk", "litres/head/day", "kg milk solids/head/day")</f>
         <v>litres/head/day</v>
       </c>
+      <c r="R50" s="7"/>
+    </row>
+    <row r="51" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E51" s="6"/>
+      <c r="F51" s="6"/>
+      <c r="R51" s="7"/>
+    </row>
+    <row r="52" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D52" s="53" t="s">
+        <v>245</v>
+      </c>
+      <c r="E52" s="40" t="s">
+        <v>242</v>
+      </c>
+      <c r="F52" s="40" t="s">
+        <v>243</v>
+      </c>
       <c r="R52" s="7"/>
     </row>
     <row r="53" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E53" s="6"/>
-      <c r="F53" s="6"/>
-      <c r="R53" s="7"/>
-    </row>
-    <row r="54" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D54" s="53" t="s">
-        <v>245</v>
-      </c>
-      <c r="E54" s="40" t="s">
-        <v>242</v>
-      </c>
-      <c r="F54" s="40" t="s">
-        <v>243</v>
-      </c>
-      <c r="R54" s="7"/>
-    </row>
-    <row r="55" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D55" s="1" t="s">
+      <c r="D53" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="E55" s="120">
+      <c r="E53" s="120">
         <f>SourceData_Dairy_FatContentInMilk_Data/100</f>
         <v>0.04</v>
       </c>
-      <c r="F55" s="128">
+      <c r="F53" s="128">
         <f>SourceData_Dairy_FatContentInMilk_Data/100</f>
         <v>0.04</v>
       </c>
-      <c r="G55" s="2" t="s">
+      <c r="G53" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="R55" s="7"/>
-    </row>
-    <row r="56" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D56" s="1" t="s">
+      <c r="R53" s="7"/>
+    </row>
+    <row r="54" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D54" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="E56" s="120">
+      <c r="E54" s="120">
         <f>SourceData_Dairy_ProteinContentInMilk_Data/100</f>
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="F56" s="128">
+      <c r="F54" s="128">
         <f>SourceData_Dairy_ProteinContentInMilk_Data/100</f>
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="G54" s="2" t="s">
         <v>244</v>
       </c>
+      <c r="R54" s="7"/>
+    </row>
+    <row r="55" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R55" s="7"/>
+    </row>
+    <row r="56" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="R56" s="7"/>
     </row>
     <row r="57" spans="4:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15558,7 +15556,7 @@
       <c r="M178" s="2"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E10:M10 E24:M25 E28:M29 E36:J37 K36:M38 E40:K41 L41:M43 K42 O43:P43 N44 J85:J90 K89:M89 K95:M95 F98 J101:J106 K105:M105 K110:M110 K114:M114 K123:M123">
+  <conditionalFormatting sqref="E10:M10 E24:M25 E28:M29 E36:J37 K36:M38 E40:K41 L41:M42 K42 O43:P43 J85:J90 K89:M89 K95:M95 F98 J101:J106 K105:M105 K110:M110 K114:M114 K123:M123">
     <cfRule type="cellIs" dxfId="6" priority="30" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -15600,7 +15598,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E110" xr:uid="{20E9D9A1-CABD-46A5-B149-02F06B30AA0E}">
       <formula1>INDIRECT("Table_SourceData_Dairy_IrrigationMethods[Irrigation method]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E62" xr:uid="{9FB53635-991F-44AA-A123-E8ABEF9EE0A6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E60" xr:uid="{9FB53635-991F-44AA-A123-E8ABEF9EE0A6}">
       <formula1>INDIRECT("Table_SourceData_Dairy_ProductionSystemTemplates[Area]")</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E79:E81 E95:E97" xr:uid="{00A4EA4C-90D3-4150-979D-4D71C7F37A31}">
@@ -15609,7 +15607,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7" xr:uid="{4AE50AD3-14AA-4BCF-9F4A-CDB83D5683F7}">
       <formula1>INDIRECT("Table_SourceData_Dairy_WjCowsHeifers[Breed]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E49" xr:uid="{2CEBE667-943C-46F8-889E-3F0627762496}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E47" xr:uid="{2CEBE667-943C-46F8-889E-3F0627762496}">
       <formula1>"Litres of milk, Milk solids"</formula1>
     </dataValidation>
   </dataValidations>
@@ -25301,21 +25299,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAXAB1ADAAMAAyADcAUgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcALAAgAGEAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAaQBzACAAYwBvAG4AcwBpAHMAdABlAG4AdABsAHkAIABcAHUAMAAwADIANwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdAFwAdQAwADAAMgA3ACAAYQBuAGQAIABpAHMAIABuAG8AdAAgAHUAcwBlAGQAIABpAG4AIABjAGEAbABjAHUAbABhAHQAaQBvAG4ALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHIAZQBlAGQAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBsAGwAIABiAHIAZQBlAGQAcwBcACIALAAgADYAMAAwACwAIAAyADIANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAVwBHAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA1ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABDAG8AdwBzAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAANQA5ADAALAAgADUAOQAwACwAIAA1ADkAMAAsACAANwA3ADAALAAgADcANwAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAdABhACAAZgBvAHIAIABwAHIAZQAgAC0AIAB3AGUAYQBuAGUAZAAgAGMAYQBsAHYAZQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBqAD0AMwAsADUAOwAgAE4AUABXAGoAPQAzACwANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzAFwAdQAwADAAMwBjADEAXAAiACwAIAAwAC4AMAAxADcANgAsACAAMAAuADIANgA4ADUALAAgADAALgAwADEAMwA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwBcAHUAMAAwADMAYwAxAFwAIgAsACAAMAAuADAAMgAwADQALAAgADAALgAzADAAMAAzACwAIAAwAC4AMAAwADkAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBDAEYAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEAMAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBUAEEAUwBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAuADcAMgAsACAAMAAuADcANgAsACAAMAAuADgALAAgADAALgA3ADgALAAgADAALgA3ADQALAAgADAALgA2ADkALAAgADAALgA3ADMALAAgADAALgA3ADYALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwAgACgAYQApAFwAIgAsACAAMAAuADEANQAsACAAMAAuADEAOAAsACAAMAAuADUAMAAsACAAMAAuADIANAAsACAAMAAuADEANwAsACAAMAAuADEAMwAsACAAMAAuADEANwAsACAAMAAuADEAOAAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAG0AOwAgAEYAcgBhAGMARwBBAFMATQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADAALgAwADEANwA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjACAAMQAgAHkAZQBhAHIAXAAiACwAIAAwAC4AMAAyADAANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBSAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA5ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABJAG4AYwByAGUAYQBzAGUAZAAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAIAAoAE0AUgBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUgBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFIAagBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMALAAgAGEAbgBkACAAaABvAHUAcwBlACAAYwBvAHcAcwBcACIALAAgADEALgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAbwB0AGgAZQByACAAYwBhAHQAdABsAGUAIABjAGwAYQBzAHMAZQBzAFwAIgAsACAAMQAuADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAdgBvAGkAZABlAGQAIAB0AG8AIABlAGEAYwBoACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAE0AUwBqAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBqAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEUAeABjAGwAdQBkAGUAZAAgAFwAdQAwADAAMgA3AEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQBcAHUAMAAwADIANwAgAHIAbwB3ACAAYQBzACAAdABoAGkAcwAgAGkAbgBmAG8AcgBtAGEAdABpAG8AbgAgAGkAcwAgAGkAbgAgAHQAaABlACAAdABhAGIAbABlACAAdABpAHQAbABlAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQByAGUAYQBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE0AaQBsAGsAaQBuAGcAIABTAGgAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAcABhAGQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMQA6ACAARwByAGEAegBlAGQAIABPAG4AbAB5AFwAIgAsACAAMAAuADgAOQAsACAAMAAuADEAMQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADIAOgAgAE8AbgAgAGYAZQBlAGQAcABhAGQAIABmAG8AcgAgAFwAdQAwADAAMwBjADEAMAAgAGgAcgAvAGQAYQB5ACAAZgBvAHIAIABcAHUAMAAwADMAYwAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMwAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEANAAgAFAAYQBzAHQAdQByAGUAXAAiACwAIAAwACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEAIABBAG4AZQByAG8AYgBpAGMAIABMAGEAZwBvAG8AbgBcACIALAAgADAALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbABcACIALAAgADAALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMwAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwBcACIALAAgADAALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQA0ACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXABuAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABmAG8AcgAgAGUAYQBjAGgAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgBwAHUAdAAgAGMAbABhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGEAeQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADIAXAB0AEQAQQBUAEEAIAAoAE0ARQBUAEgATwBEACAAMQAgAEEATgBEACAAMgAgAE8AUABUAEkATwBOAFMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBlAGUAIAB0AGUAeAB0ACAAaQBuACAAZABvAGMAdQBtAGUAbgB0ACAAdABvACAAdABhAGIAbABlACwAIABtAGEAdABjAGgAaQBuAGcAIABsAGkAdgBlAHMAdABvAGMAawAgAGMAbABhAHMAcwAgAG4AYQBtAGUAcwAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEQAdQByAGEAdABpAG8AbgAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHAAcgBlAC0AdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMAXAAiACwAIAAzADYANQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAgADEAIAB5AGUAYQByAFwAIgAsACAAMgA4ADEALAAgADgANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAgADEAIAB5AGUAYQByAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBEAGUAZgBhAHUAbAB0ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAB3AGgAZQBuACAAbQBhAG4AdQByAGUAIABpAHMAIABlAHgAYwByAGUAdABlAGQAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQAuACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAZQBmAGEAdQBsAHQAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAHcAaABlAG4AIABtAGEAbgB1AHIAZQAgAGkAcwAgAGUAeABjAHIAZQB0AGUAZAAgAHQAbwAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawAgACgAbQA9ADEANAApAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAyADQAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4ARgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBDAF8AagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQALgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAFwAbgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADIAIABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAzACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcARABQAFcAXAB1ADAAMAAyADcAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABoAGEAbgBkAGwAaQBuAGcAIABvAGYAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAZAB1AHIAYQB0AGkAbwBuAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXABuAE0AXwBqAFwAbgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ASQBfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABJAF8AagAsAFwAbgAgACAAIAAgADIAMAAuADcAIAAqACAASQBfAGoAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGgAYQByAG0AbABlAHkAIABlAHQAIABhAGwALgAgACgAMgAwADEANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADMAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4ARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgBJAF8AagBcAG4AawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAbgBXAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQBcAG4ATABXAEcAXwBqACAAPQAgAGwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATQBSAF8AagAgAD0AIABpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ATQBJAF8AagAgAD0AIABhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABXAF8AagAsACAATABXAEcAXwBqACwAIABNAFIAXwBqACwAIABNAEkAXwBqACwAXABuACAAIAAgACAAKAAxAC4AMQA4ADUAIAArACAAMAAuADAAMAA0ADUANAAgACoAIABXAF8AagAgAC0AIAAwAC4AMAAwADAAMAAwADIANgAgACoAIABXAF8AagAgAF4AIAAyACAAKwAgADAALgAzADEANQAgACoAIABMAFcARwBfAGoAKQAgAF4AIAAyACAAKgAgAE0AUgBfAGoAIAArACAATQBJAF8AagBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0AFwAIgAsACAAXAAiAGsAZwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAVwBHAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgBcACIALAAgAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFIAXwBqAFwAIgAsACAAXAAiAGkAbgBjAHIAZQBhAHMAZQAgAGkAbgAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBJAF8AagBcACIALAAgAFwAIgBhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAE0ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBJAF8AagA9ACgATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFACkALwAoAEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqACkAXABuAE0AUABfAGoAIAA9ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAEwALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATgBFACAAPQAgAG4AZQB0ACAAZQBuAGUAcgBnAHkAIAAoAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrACkAXABuAEcARQBDACAAPQAgAGcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgACgATQBKAC8AawBnAEQATQApAFwAbgBrACAAPQAgAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgBxAG0AXwBqACAAPQAgAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFAAXwBqACwAIABOAEUALAAgAEcARQBDACwAIABrACwAIABxAG0AXwBqACwAXABuACAAIAAgACAAKABNAFAAXwBqACAAKgAgADEALgAwADMAIAAqACAATgBFACkAIAAvACAAKABHAEUAQwAgACoAIABrACAAKgAgAHEAbQBfAGoAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADQAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAD0AXABcAGYAcgBhAGMAewBNAFAAXwBqAFwAXAB0AGkAbQBlAHMAIAAxAC4AMAAzAFwAXAB0AGkAbQBlAHMAIABOAEUAfQB7AEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAXwBqAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABpAGYAIABpAG4AcAB1AHQAIABhAHMAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsAKQBcACIALAAgAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBFAFwAIgAsACAAXAAiAG4AZQB0ACAAZQBuAGUAcgBnAHkAXAAiACwAIABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAvAGsAZwAgAG0AaQBsAGsAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEUAQwBcACIALAAgAFwAIgBnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAXAAiACwAIABcACIATQBKAC8AawBnAEQATQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGsAXAAiACwAIABcACIAZQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAG0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUAIABlAG4AZQByAGcAeQAgAHUAcwBlACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAG0AXwBqAFwAIgAsACAAXAAiAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgANgApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAFwAbgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcAG4ATQBQAF8AagBcAG4ATAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBQAF8AagA9AE0AUwBfAGoALwAoADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQApAFwAbgBNAFMAXwBqACAAPQAgAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIAAoAGsAZwAgAE0AUwAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBGAEMAXwBqACAAPQAgAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4AUABDAF8AagAgAD0AIABwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFMAXwBqACwAIABGAEMAXwBqACwAIABQAEMAXwBqACwAXABuACAAIAAgACAATQBTAF8AagAgAC8AIAAoADAALgAwADEAIAAqACAAKABGAEMAXwBqACAAKwAgAFAAQwBfAGoAKQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAYwBvAG4AdgBlAHIAdABlAGQAIABmAHIAbwBtACAAbQBpAGwAawAgAHMAbwBsAGkAZABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagA9AFwAXABmAHIAYQBjAHsATQBTAF8AagB9AHsAMAAuADAAMQBcAFwAdABpAG0AZQBzACAAKABGAEMAXwBqACsAUABDAF8AagApAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAGkAbgBwAHUAdAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdAAgAHYAYQByAGkAYQBiAGwAZQAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAdQBzAGUAIABvAGYAIABlAGkAdABoAGUAcgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwAgAG8AcgAgAGwAaQB0AHIAZQBzACAAbwBmACAAbQBpAGwAawAuACAAQwBvAG4AdgBlAHIAdABlAGQAIABpAG4AcAB1AHQAIABGAEMAIABhAG4AZAAgAFAAQwAgAHAAZQByAGMAZQBuAHQAIAB0AG8AIABpAG4AdABlAGcAZQByAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQAgAG8AZgAgAGQAaQBlAHQAXABuAHEAbQBfAGoAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4AcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcAG4ARABNAEQAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQATQBEAF8AagAsAFwAbgAgACAAIAAgADAALgA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABNAEQAXwBqACwAXABuACAAIAAgACAAMAAuADAAMAA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBxAG0AXwBqAD0AMAAuADAAMAA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABjAGgAYQBuAGcAZQBkACAAMAAuADcAOQA1ACAAdABvACAAMAAuADAAMAA3ADkANQAgAHcAaABpAGMAaAAgAGkAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAdQBzAGUAZAAgAGkAbgAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdABcACIAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBEAGEAaQByAHkAIgAsACIAdABlAHgAdAAiADoAIgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAE0ATQBTAEEAZgB0AGUAcgBTAG8AbABpAGQAUwBlAHAAYQByAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAsACAARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAgACoAIAAoAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAtACgATQBNAFMARgByAGEAYwB0AGkAbwBuACoARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACkAKQBcAG4AKQA7AFwAbgBcAG4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAsAFwAbgAgACAAIAAgAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMgBTAGUAcABhAHIAYQB0AGUAZAAsACAAXABuACAAIAAgACAATQBNAFMAMwBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgAXABuACAAIAAgACAAIAAgACAAIABJAG4AaQB0AGEAbABTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBGAHIAYQBjAHQAaQBvAG4AIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAxAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAzAFMAZQBwAGEAcgBhAHQAZQBkACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -25510,35 +25502,30 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAXAB1ADAAMAAyADcAUgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcALAAgAGEAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAaQBzACAAYwBvAG4AcwBpAHMAdABlAG4AdABsAHkAIABcAHUAMAAwADIANwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdAFwAdQAwADAAMgA3ACAAYQBuAGQAIABpAHMAIABuAG8AdAAgAHUAcwBlAGQAIABpAG4AIABjAGEAbABjAHUAbABhAHQAaQBvAG4ALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHIAZQBlAGQAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAEMAbwB3AHMAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIASABlAGkAZgBlAHIAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBsAGwAIABiAHIAZQBlAGQAcwBcACIALAAgADYAMAAwACwAIAAyADIANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AIAAoAGsAZwApACAAKABMAFcARwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAVwBHAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA1ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABDAG8AdwBzAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAxACAAKAB3AGUAYQBuAGUAZAApAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBlADEAXAAiACwAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAMQBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAANQA5ADAALAAgADUAOQAwACwAIAA1ADkAMAAsACAANwA3ADAALAAgADcANwAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAdABhACAAZgBvAHIAIABwAHIAZQAgAC0AIAB3AGUAYQBuAGUAZAAgAGMAYQBsAHYAZQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBqAD0AMwAsADUAOwAgAE4AUABXAGoAPQAzACwANQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzAFwAdQAwADAAMwBjADEAXAAiACwAIAAwAC4AMAAxADcANgAsACAAMAAuADIANgA4ADUALAAgADAALgAwADEAMwA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwBcAHUAMAAwADMAYwAxAFwAIgAsACAAMAAuADAAMgAwADQALAAgADAALgAzADAAMAAzACwAIAAwAC4AMAAwADkAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBDAEYAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA2AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADEAMAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBUAEEAUwBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAuADcAMgAsACAAMAAuADcANgAsACAAMAAuADgALAAgADAALgA3ADgALAAgADAALgA3ADQALAAgADAALgA2ADkALAAgADAALgA3ADMALAAgADAALgA3ADYALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgAC0AIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwAgACgAYQApAFwAIgAsACAAMAAuADEANQAsACAAMAAuADEAOAAsACAAMAAuADUAMAAsACAAMAAuADIANAAsACAAMAAuADEANwAsACAAMAAuADEAMwAsACAAMAAuADEANwAsACAAMAAuADEAOAAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIABhAG4AZAAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAG0AOwAgAEYAcgBhAGMARwBBAFMATQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA3AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADAALgAwADEANwA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAFwAdQAwADAAMwBjACAAMQAgAHkAZQBhAHIAXAAiACwAIAAwAC4AMAAyADAANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBSAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA5ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABJAG4AYwByAGUAYQBzAGUAZAAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAIAAoAE0AUgBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUgBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFIAagBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMALAAgAGEAbgBkACAAaABvAHUAcwBlACAAYwBvAHcAcwBcACIALAAgADEALgAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAbwB0AGgAZQByACAAYwBhAHQAdABsAGUAIABjAGwAYQBzAHMAZQBzAFwAIgAsACAAMQAuADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAdgBvAGkAZABlAGQAIAB0AG8AIABlAGEAYwBoACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAE0AUwBqAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBqAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEUAeABjAGwAdQBkAGUAZAAgAFwAdQAwADAAMgA3AEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQBcAHUAMAAwADIANwAgAHIAbwB3ACAAYQBzACAAdABoAGkAcwAgAGkAbgBmAG8AcgBtAGEAdABpAG8AbgAgAGkAcwAgAGkAbgAgAHQAaABlACAAdABhAGIAbABlACAAdABpAHQAbABlAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQByAGUAYQBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE0AaQBsAGsAaQBuAGcAIABTAGgAZQBkAFwAIgAsACAAXAAiAEYAZQBlAGQAcABhAGQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMQA6ACAARwByAGEAegBlAGQAIABPAG4AbAB5AFwAIgAsACAAMAAuADgAOQAsACAAMAAuADEAMQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADIAOgAgAE8AbgAgAGYAZQBlAGQAcABhAGQAIABmAG8AcgAgAFwAdQAwADAAMwBjADEAMAAgAGgAcgAvAGQAYQB5ACAAZgBvAHIAIABcAHUAMAAwADMAYwAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMwAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AXAAiACwAIABcACIATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEANAAgAFAAYQBzAHQAdQByAGUAXAAiACwAIAAwACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADEAIABBAG4AZQByAG8AYgBpAGMAIABMAGEAZwBvAG8AbgBcACIALAAgADAALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbABcACIALAAgADAALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0AMwAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkADoAIABEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAcwBcACIALAAgADAALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQA0ACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXABuAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABmAG8AcgAgAGUAYQBjAGgAIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAGkAbgBwAHUAdAAgAGMAbABhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGEAeQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADIAXAB0AEQAQQBUAEEAIAAoAE0ARQBUAEgATwBEACAAMQAgAEEATgBEACAAMgAgAE8AUABUAEkATwBOAFMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABDAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBlAGUAIAB0AGUAeAB0ACAAaQBuACAAZABvAGMAdQBtAGUAbgB0ACAAdABvACAAdABhAGIAbABlACwAIABtAGEAdABjAGgAaQBuAGcAIABsAGkAdgBlAHMAdABvAGMAawAgAGMAbABhAHMAcwAgAG4AYQBtAGUAcwAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEQAdQByAGEAdABpAG8AbgAgACgAdwBlAGEAbgBlAGQAKQBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHAAcgBlAC0AdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGwAawBpAG4AZwAgAGMAbwB3AHMAXAAiACwAIAAzADYANQAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAXAB1ADAAMAAzAGUAIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIABcAHUAMAAwADMAYwAgADEAIAB5AGUAYQByAFwAIgAsACAAMgA4ADEALAAgADgANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbABsAHMAIABcAHUAMAAwADMAZQAgADEAIAB5AGUAYQByAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAXAB1ADAAMAAzAGMAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAG8AcgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABNAE0AUwAgAG8AbgBsAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBEAGUAZgBhAHUAbAB0ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAB3AGgAZQBuACAAbQBhAG4AdQByAGUAIABpAHMAIABlAHgAYwByAGUAdABlAGQAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQAuACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAZQBmAGEAdQBsAHQAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAHcAaABlAG4AIABtAGEAbgB1AHIAZQAgAGkAcwAgAGUAeABjAHIAZQB0AGUAZAAgAHQAbwAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawAgACgAbQA9ADEANAApAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAF8ATABFAEEAQwBIAF8ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAyADQAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4ARgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBDAF8AagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQALgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAFwAbgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADIAIABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAzACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcARABQAFcAXAB1ADAAMAAyADcAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABoAGEAbgBkAGwAaQBuAGcAIABvAGYAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAZAB1AHIAYQB0AGkAbwBuAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXABuAE0AXwBqAFwAbgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ASQBfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABJAF8AagAsAFwAbgAgACAAIAAgADIAMAAuADcAIAAqACAASQBfAGoAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGgAYQByAG0AbABlAHkAIABlAHQAIABhAGwALgAgACgAMgAwADEANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAPQAyADAALgA3AFwAXAB0AGkAbQBlAHMAIABJAF8AagBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADMAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4ARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgBJAF8AagBcAG4AawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAbgBXAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQBcAG4ATABXAEcAXwBqACAAPQAgAGwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATQBSAF8AagAgAD0AIABpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ATQBJAF8AagAgAD0AIABhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABXAF8AagAsACAATABXAEcAXwBqACwAIABNAFIAXwBqACwAIABNAEkAXwBqACwAXABuACAAIAAgACAAKAAxAC4AMQA4ADUAIAArACAAMAAuADAAMAA0ADUANAAgACoAIABXAF8AagAgAC0AIAAwAC4AMAAwADAAMAAwADIANgAgACoAIABXAF8AagAgAF4AIAAyACAAKwAgADAALgAzADEANQAgACoAIABMAFcARwBfAGoAKQAgAF4AIAAyACAAKgAgAE0AUgBfAGoAIAArACAATQBJAF8AagBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAF8AagA9ACgAMQAuADEAOAA1ACsAMAAuADAAMAA0ADUANABcAFwAdABpAG0AZQBzACAAVwBfAGoALQAwAC4AMAAwADAAMAAwADIANgBcAFwAdABpAG0AZQBzACAAVwBfAGoAXgAyACsAMAAuADMAMQA1AFwAXAB0AGkAbQBlAHMAIABMAFcARwBfAGoAKQBeADIAXABcAHQAaQBtAGUAcwAgAE0AUgBfAGoAKwBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0AFwAIgAsACAAXAAiAGsAZwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAVwBHAF8AagBcACIALAAgAFwAIgBsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgBcACIALAAgAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFIAXwBqAFwAIgAsACAAXAAiAGkAbgBjAHIAZQBhAHMAZQAgAGkAbgAgAG0AZQB0AGEAYgBvAGwAaQBjACAAcgBhAHQAZQAgAHcAaABlAG4AIABwAHIAbwBkAHUAYwBpAG4AZwAgAG0AaQBsAGsAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBJAF8AagBcACIALAAgAFwAIgBhAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAE0ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBJAF8AagA9ACgATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFACkALwAoAEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqACkAXABuAE0AUABfAGoAIAA9ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAEwALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATgBFACAAPQAgAG4AZQB0ACAAZQBuAGUAcgBnAHkAIAAoAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrACkAXABuAEcARQBDACAAPQAgAGcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgACgATQBKAC8AawBnAEQATQApAFwAbgBrACAAPQAgAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgBxAG0AXwBqACAAPQAgAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAIAAoAGYAcgBhAGMAdABpAG8AbgApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFAAXwBqACwAIABOAEUALAAgAEcARQBDACwAIABrACwAIABxAG0AXwBqACwAXABuACAAIAAgACAAKABNAFAAXwBqACAAKgAgADEALgAwADMAIAAqACAATgBFACkAIAAvACAAKABHAEUAQwAgACoAIABrACAAKgAgAHEAbQBfAGoAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADQAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEkAXwBqAD0AXABcAGYAcgBhAGMAewBNAFAAXwBqAFwAXAB0AGkAbQBlAHMAIAAxAC4AMAAzAFwAXAB0AGkAbQBlAHMAIABOAEUAfQB7AEcARQBDAFwAXAB0AGkAbQBlAHMAIABrAFwAXAB0AGkAbQBlAHMAIABxAG0AXwBqAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAXwBqAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABpAGYAIABpAG4AcAB1AHQAIABhAHMAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsAKQBcACIALAAgAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBFAFwAIgAsACAAXAAiAG4AZQB0ACAAZQBuAGUAcgBnAHkAXAAiACwAIABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAvAGsAZwAgAG0AaQBsAGsAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEUAQwBcACIALAAgAFwAIgBnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAXAAiACwAIABcACIATQBKAC8AawBnAEQATQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGsAXAAiACwAIABcACIAZQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAG0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUAIABlAG4AZQByAGcAeQAgAHUAcwBlACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAG0AXwBqAFwAIgAsACAAXAAiAG0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIAB0AGgAZQAgAGQAaQBlAHQAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgANgApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAFwAbgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcAG4ATQBQAF8AagBcAG4ATAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATQBQAF8AagA9AE0AUwBfAGoALwAoADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQApAFwAbgBNAFMAXwBqACAAPQAgAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIAAoAGsAZwAgAE0AUwAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBGAEMAXwBqACAAPQAgAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4AUABDAF8AagAgAD0AIABwAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAFMAXwBqACwAIABGAEMAXwBqACwAIABQAEMAXwBqACwAXABuACAAIAAgACAATQBTAF8AagAgAC8AIAAoADAALgAwADEAIAAqACAAKABGAEMAXwBqACAAKwAgAFAAQwBfAGoAKQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAYwBvAG4AdgBlAHIAdABlAGQAIABmAHIAbwBtACAAbQBpAGwAawAgAHMAbwBsAGkAZABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBQAF8AagA9AFwAXABmAHIAYQBjAHsATQBTAF8AagB9AHsAMAAuADAAMQBcAFwAdABpAG0AZQBzACAAKABGAEMAXwBqACsAUABDAF8AagApAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAGkAbgBwAHUAdAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABVAFwAIgAsACAAXAAiAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUwBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIALAAgAFwAIgBrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAEMAXwBqAFwAIgAsACAAXAAiAGYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAQwBfAGoAXAAiACwAIABcACIAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAdQBuAGkAdAAgAHYAYQByAGkAYQBiAGwAZQAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAdQBzAGUAIABvAGYAIABlAGkAdABoAGUAcgAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwAgAG8AcgAgAGwAaQB0AHIAZQBzACAAbwBmACAAbQBpAGwAawAuACAAQwBvAG4AdgBlAHIAdABlAGQAIABpAG4AcAB1AHQAIABGAEMAIABhAG4AZAAgAFAAQwAgAHAAZQByAGMAZQBuAHQAIAB0AG8AIABpAG4AdABlAGcAZQByAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQAgAG8AZgAgAGQAaQBlAHQAXABuAHEAbQBfAGoAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4AcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcAG4ARABNAEQAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQATQBEAF8AagAsAFwAbgAgACAAIAAgADAALgA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABNAEQAXwBqACwAXABuACAAIAAgACAAMAAuADAAMAA3ADkANQAgACoAIAAoAEQATQBEAF8AagAgACoAIAAxADAAMAApACAALQAgADAALgAwADAAMQA0AFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBxAG0AXwBqAD0AMAAuADAAMAA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABjAGgAYQBuAGcAZQBkACAAMAAuADcAOQA1ACAAdABvACAAMAAuADAAMAA3ADkANQAgAHcAaABpAGMAaAAgAGkAcwAgAHQAaABlACAAdgBhAGwAdQBlACAAdQBzAGUAZAAgAGkAbgAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdABcACIAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBEAGEAaQByAHkAIgAsACIAdABlAHgAdAAiADoAIgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAE0ATQBTAEEAZgB0AGUAcgBTAG8AbABpAGQAUwBlAHAAYQByAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAsACAARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAgACoAIAAoAE0ATQBTAEYAcgBhAGMAdABpAG8AbgAtACgATQBNAFMARgByAGEAYwB0AGkAbwBuACoARgByAGEAYwB0AGkAbwBuAFMAZQBwAGEAcgBhAHQAZQBkACkAKQBcAG4AKQA7AFwAbgBcAG4AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAsAFwAbgAgACAAIAAgAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMgBTAGUAcABhAHIAYQB0AGUAZAAsACAAXABuACAAIAAgACAATQBNAFMAMwBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgAXABuACAAIAAgACAAIAAgACAAIABJAG4AaQB0AGEAbABTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBGAHIAYQBjAHQAaQBvAG4AIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAxAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAxAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAyAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAKABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAgACoAIABNAE0AUwAzAFMAZQBwAGEAcgBhAHQAZQBkACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFAAaQBnAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25557,10 +25544,21 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix false-negative in phantom external-link detection; clean up 4 missed workbooks
remove-phantom-external-links.ps1's usage check matched a bare [N] substring
anywhere in worksheet/workbook XML, so source-citation text baked into LAMBDA
description strings ("Dairy Australia [1]", "IPCC (2019), Chapter 10 [4]")
false-positived as a live reference and hid a genuinely phantom
Common_v03.xlsx link in 13_Scope3_WIP_v14.xlsx, 3_3_Enteric_Dairy_WIP_v04.xlsx,
4_2_ManureManagement_BeefPasture_WIP_v10.xlsx and
4_3_ManureManagement_Dairy_WIP_v12.xlsx - these kept reporting the external
link even after the prior self-heal fix. Detection (and the renumber pass,
same latent risk) now requires genuine external-reference syntax via
lookaround ([N]!Name, [N]SheetName!, '[N]Sheet Name'!) instead of a bare
bracketed number. Removed the 4 confirmed phantom links; find-excel-errors.ps1
confirms all four clean.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
+++ b/Excel/3_3_Enteric_Dairy_WIP_v04.xlsx
@@ -24,9 +24,6 @@
     <sheet name="Constants - Common Livestock" sheetId="43" r:id="rId9"/>
     <sheet name="Acknowledgements" sheetId="72" r:id="rId10"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId11"/>
-  </externalReferences>
   <definedNames>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -9337,26 +9334,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Home"/>
-      <sheetName val="Constants - Common"/>
-      <sheetName val="Acknowledgements"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>

</xml_diff>